<commit_message>
Bottom PCB BOMs updated according to the recent schematic changes.
</commit_message>
<xml_diff>
--- a/Deliverables/SM_Bottom Board/_BOM/SM_Bottom_Board_LCSC.xlsx
+++ b/Deliverables/SM_Bottom Board/_BOM/SM_Bottom_Board_LCSC.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark\ColeBenson-SmartMotors\Deliverables\SM_Bottom Board\_BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72E71F20-2E3E-4FE2-9054-80863632ACC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{138D62B4-CD82-41E0-9D1B-6ED06D1F076E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="780" yWindow="780" windowWidth="10335" windowHeight="10620" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SM_Bottom_Board" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="251" uniqueCount="202">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="243" uniqueCount="197">
   <si>
     <t>Description</t>
   </si>
@@ -306,30 +306,9 @@
     <t>RC0603FR-07470RL</t>
   </si>
   <si>
-    <t>46R6</t>
-  </si>
-  <si>
-    <t>Res SMD 0603 46.4 Ohm 1% 1/10W</t>
-  </si>
-  <si>
     <t>R7, R8</t>
   </si>
   <si>
-    <t>Panasonic</t>
-  </si>
-  <si>
-    <t>ERJ-3EKF46R4V</t>
-  </si>
-  <si>
-    <t>RES SMD 1K OHM 1% 1/20W 0201</t>
-  </si>
-  <si>
-    <t>R9, R10</t>
-  </si>
-  <si>
-    <t>RC0201FR-071KL</t>
-  </si>
-  <si>
     <t>B3U-1000P</t>
   </si>
   <si>
@@ -609,12 +588,6 @@
     <t>C114669</t>
   </si>
   <si>
-    <t>C403240</t>
-  </si>
-  <si>
-    <t>C138165</t>
-  </si>
-  <si>
     <t>C231329</t>
   </si>
   <si>
@@ -634,6 +607,18 @@
   </si>
   <si>
     <t>Not available</t>
+  </si>
+  <si>
+    <t>Res SMD 0603 57.6Ohm 1% 1/10W</t>
+  </si>
+  <si>
+    <t>RC0603FR-0757R6L</t>
+  </si>
+  <si>
+    <t>C245984</t>
+  </si>
+  <si>
+    <t>57R6</t>
   </si>
 </sst>
 </file>
@@ -1036,7 +1021,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="63">
+  <cellXfs count="64">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1148,6 +1133,54 @@
     <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="9" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="9" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="9" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="12" fillId="4" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="4" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="14" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="14" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="4" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="10" fillId="4" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -1172,53 +1205,8 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="9" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="9" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="9" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="12" fillId="4" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="6" fillId="4" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="14" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="14" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="6" fillId="4" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="10" fillId="4" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="6" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1504,7 +1492,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:S34"/>
+  <dimension ref="A1:S33"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.140625" bestFit="1" customWidth="1"/>
@@ -1529,34 +1517,34 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:19" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="43" t="s">
-        <v>159</v>
-      </c>
-      <c r="B1" s="44"/>
-      <c r="C1" s="44"/>
-      <c r="D1" s="44"/>
-      <c r="E1" s="44"/>
-      <c r="F1" s="44"/>
-      <c r="G1" s="44"/>
-      <c r="H1" s="44"/>
-      <c r="I1" s="44"/>
-      <c r="J1" s="44"/>
-      <c r="K1" s="44"/>
-      <c r="L1" s="44"/>
-      <c r="M1" s="44"/>
-      <c r="N1" s="44"/>
-      <c r="O1" s="44"/>
-      <c r="P1" s="44"/>
-      <c r="Q1" s="44"/>
-      <c r="R1" s="44"/>
-      <c r="S1" s="45"/>
+      <c r="A1" s="59" t="s">
+        <v>152</v>
+      </c>
+      <c r="B1" s="60"/>
+      <c r="C1" s="60"/>
+      <c r="D1" s="60"/>
+      <c r="E1" s="60"/>
+      <c r="F1" s="60"/>
+      <c r="G1" s="60"/>
+      <c r="H1" s="60"/>
+      <c r="I1" s="60"/>
+      <c r="J1" s="60"/>
+      <c r="K1" s="60"/>
+      <c r="L1" s="60"/>
+      <c r="M1" s="60"/>
+      <c r="N1" s="60"/>
+      <c r="O1" s="60"/>
+      <c r="P1" s="60"/>
+      <c r="Q1" s="60"/>
+      <c r="R1" s="60"/>
+      <c r="S1" s="61"/>
     </row>
     <row r="2" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>146</v>
+        <v>139</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>147</v>
+        <v>140</v>
       </c>
       <c r="C2" s="5" t="s">
         <v>0</v>
@@ -1565,7 +1553,7 @@
         <v>1</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>148</v>
+        <v>141</v>
       </c>
       <c r="F2" s="5" t="s">
         <v>3</v>
@@ -1574,48 +1562,48 @@
         <v>2</v>
       </c>
       <c r="H2" s="5" t="s">
+        <v>142</v>
+      </c>
+      <c r="I2" s="5" t="s">
+        <v>166</v>
+      </c>
+      <c r="J2" s="5" t="s">
+        <v>143</v>
+      </c>
+      <c r="K2" s="5" t="s">
+        <v>167</v>
+      </c>
+      <c r="L2" s="5" t="s">
+        <v>144</v>
+      </c>
+      <c r="M2" s="5" t="s">
+        <v>145</v>
+      </c>
+      <c r="N2" s="5" t="s">
+        <v>146</v>
+      </c>
+      <c r="O2" s="5" t="s">
+        <v>147</v>
+      </c>
+      <c r="P2" s="5" t="s">
+        <v>148</v>
+      </c>
+      <c r="Q2" s="5" t="s">
         <v>149</v>
       </c>
-      <c r="I2" s="5" t="s">
-        <v>173</v>
-      </c>
-      <c r="J2" s="5" t="s">
+      <c r="R2" s="5" t="s">
         <v>150</v>
       </c>
-      <c r="K2" s="5" t="s">
-        <v>174</v>
-      </c>
-      <c r="L2" s="5" t="s">
+      <c r="S2" s="5" t="s">
         <v>151</v>
-      </c>
-      <c r="M2" s="5" t="s">
-        <v>152</v>
-      </c>
-      <c r="N2" s="5" t="s">
-        <v>153</v>
-      </c>
-      <c r="O2" s="5" t="s">
-        <v>154</v>
-      </c>
-      <c r="P2" s="5" t="s">
-        <v>155</v>
-      </c>
-      <c r="Q2" s="5" t="s">
-        <v>156</v>
-      </c>
-      <c r="R2" s="5" t="s">
-        <v>157</v>
-      </c>
-      <c r="S2" s="5" t="s">
-        <v>158</v>
       </c>
     </row>
     <row r="3" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="7">
         <v>1</v>
       </c>
-      <c r="B3" s="41" t="s">
-        <v>160</v>
+      <c r="B3" s="57" t="s">
+        <v>153</v>
       </c>
       <c r="C3" s="8" t="s">
         <v>5</v>
@@ -1634,7 +1622,7 @@
       </c>
       <c r="H3" s="28"/>
       <c r="I3" s="28" t="s">
-        <v>175</v>
+        <v>168</v>
       </c>
       <c r="J3" s="9" t="s">
         <v>4</v>
@@ -1650,7 +1638,7 @@
         <v>5</v>
       </c>
       <c r="N3" s="35" t="s">
-        <v>169</v>
+        <v>162</v>
       </c>
       <c r="O3" s="11">
         <v>2.5899999999999999E-2</v>
@@ -1672,7 +1660,7 @@
       <c r="A4" s="7">
         <v>2</v>
       </c>
-      <c r="B4" s="46"/>
+      <c r="B4" s="62"/>
       <c r="C4" s="12" t="s">
         <v>11</v>
       </c>
@@ -1690,7 +1678,7 @@
       </c>
       <c r="H4" s="29"/>
       <c r="I4" s="29" t="s">
-        <v>176</v>
+        <v>169</v>
       </c>
       <c r="J4" s="13" t="s">
         <v>10</v>
@@ -1702,11 +1690,11 @@
         <v>22</v>
       </c>
       <c r="M4" s="14">
-        <f t="shared" ref="M4:M32" si="0">L4*5</f>
+        <f t="shared" ref="M4:M31" si="0">L4*5</f>
         <v>110</v>
       </c>
       <c r="N4" s="35" t="s">
-        <v>169</v>
+        <v>162</v>
       </c>
       <c r="O4" s="15">
         <v>4.0000000000000001E-3</v>
@@ -1728,7 +1716,7 @@
       <c r="A5" s="7">
         <v>3</v>
       </c>
-      <c r="B5" s="46"/>
+      <c r="B5" s="62"/>
       <c r="C5" s="12" t="s">
         <v>15</v>
       </c>
@@ -1760,7 +1748,7 @@
         <v>5</v>
       </c>
       <c r="N5" s="35" t="s">
-        <v>177</v>
+        <v>170</v>
       </c>
       <c r="O5" s="15">
         <v>0.23400000000000001</v>
@@ -1773,7 +1761,7 @@
         <v>0.23400000000000001</v>
       </c>
       <c r="R5" s="15">
-        <f t="shared" ref="R5:R32" si="1">Q5*M5</f>
+        <f t="shared" ref="R5:R31" si="1">Q5*M5</f>
         <v>1.1700000000000002</v>
       </c>
       <c r="S5" s="32"/>
@@ -1782,7 +1770,7 @@
       <c r="A6" s="7">
         <v>4</v>
       </c>
-      <c r="B6" s="46"/>
+      <c r="B6" s="62"/>
       <c r="C6" s="12" t="s">
         <v>20</v>
       </c>
@@ -1800,7 +1788,7 @@
       </c>
       <c r="H6" s="14"/>
       <c r="I6" s="14" t="s">
-        <v>178</v>
+        <v>171</v>
       </c>
       <c r="J6" s="13" t="s">
         <v>19</v>
@@ -1816,7 +1804,7 @@
         <v>10</v>
       </c>
       <c r="N6" s="35" t="s">
-        <v>169</v>
+        <v>162</v>
       </c>
       <c r="O6" s="15">
         <v>3.9300000000000002E-2</v>
@@ -1838,7 +1826,7 @@
       <c r="A7" s="7">
         <v>5</v>
       </c>
-      <c r="B7" s="46"/>
+      <c r="B7" s="62"/>
       <c r="C7" s="12" t="s">
         <v>26</v>
       </c>
@@ -1855,10 +1843,10 @@
         <v>30</v>
       </c>
       <c r="H7" s="14" t="s">
-        <v>180</v>
+        <v>173</v>
       </c>
       <c r="I7" s="14" t="s">
-        <v>179</v>
+        <v>172</v>
       </c>
       <c r="J7" s="13" t="s">
         <v>25</v>
@@ -1874,7 +1862,7 @@
         <v>20</v>
       </c>
       <c r="N7" s="35" t="s">
-        <v>169</v>
+        <v>162</v>
       </c>
       <c r="O7" s="15">
         <v>2.5999999999999999E-3</v>
@@ -1896,7 +1884,7 @@
       <c r="A8" s="7">
         <v>6</v>
       </c>
-      <c r="B8" s="42"/>
+      <c r="B8" s="58"/>
       <c r="C8" s="16" t="s">
         <v>32</v>
       </c>
@@ -1914,7 +1902,7 @@
       </c>
       <c r="H8" s="30"/>
       <c r="I8" s="30" t="s">
-        <v>181</v>
+        <v>174</v>
       </c>
       <c r="J8" s="17" t="s">
         <v>31</v>
@@ -1930,7 +1918,7 @@
         <v>5</v>
       </c>
       <c r="N8" s="35" t="s">
-        <v>169</v>
+        <v>162</v>
       </c>
       <c r="O8" s="19">
         <v>3.1800000000000002E-2</v>
@@ -1952,8 +1940,8 @@
       <c r="A9" s="7">
         <v>7</v>
       </c>
-      <c r="B9" s="41" t="s">
-        <v>161</v>
+      <c r="B9" s="57" t="s">
+        <v>154</v>
       </c>
       <c r="C9" s="8" t="s">
         <v>36</v>
@@ -1972,7 +1960,7 @@
       </c>
       <c r="H9" s="10"/>
       <c r="I9" s="10" t="s">
-        <v>182</v>
+        <v>175</v>
       </c>
       <c r="J9" s="9"/>
       <c r="K9" s="9">
@@ -1986,7 +1974,7 @@
         <v>10</v>
       </c>
       <c r="N9" s="35" t="s">
-        <v>169</v>
+        <v>162</v>
       </c>
       <c r="O9" s="20">
         <v>0.13100000000000001</v>
@@ -2008,7 +1996,7 @@
       <c r="A10" s="7">
         <v>8</v>
       </c>
-      <c r="B10" s="46"/>
+      <c r="B10" s="62"/>
       <c r="C10" s="12" t="s">
         <v>41</v>
       </c>
@@ -2038,7 +2026,7 @@
         <v>5</v>
       </c>
       <c r="N10" s="35" t="s">
-        <v>172</v>
+        <v>165</v>
       </c>
       <c r="O10" s="15">
         <f>2.55/20</f>
@@ -2060,7 +2048,7 @@
       <c r="A11" s="7">
         <v>9</v>
       </c>
-      <c r="B11" s="42"/>
+      <c r="B11" s="58"/>
       <c r="C11" s="16" t="s">
         <v>55</v>
       </c>
@@ -2077,10 +2065,10 @@
         <v>58</v>
       </c>
       <c r="H11" s="36" t="s">
-        <v>183</v>
+        <v>176</v>
       </c>
       <c r="I11" s="36" t="s">
-        <v>184</v>
+        <v>177</v>
       </c>
       <c r="J11" s="17"/>
       <c r="K11" s="17">
@@ -2094,7 +2082,7 @@
         <v>5</v>
       </c>
       <c r="N11" s="37" t="s">
-        <v>169</v>
+        <v>162</v>
       </c>
       <c r="O11" s="38">
         <v>7.5800000000000006E-2</v>
@@ -2117,7 +2105,7 @@
         <v>10</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>162</v>
+        <v>155</v>
       </c>
       <c r="C12" s="21" t="s">
         <v>50</v>
@@ -2136,7 +2124,7 @@
       </c>
       <c r="H12" s="23"/>
       <c r="I12" s="23" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
       <c r="J12" s="22"/>
       <c r="K12" s="22">
@@ -2150,7 +2138,7 @@
         <v>5</v>
       </c>
       <c r="N12" s="35" t="s">
-        <v>169</v>
+        <v>162</v>
       </c>
       <c r="O12" s="24">
         <v>7.7600000000000002E-2</v>
@@ -2173,7 +2161,7 @@
         <v>11</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>163</v>
+        <v>156</v>
       </c>
       <c r="C13" s="21" t="s">
         <v>64</v>
@@ -2192,7 +2180,7 @@
       </c>
       <c r="H13" s="23"/>
       <c r="I13" s="23" t="s">
-        <v>186</v>
+        <v>179</v>
       </c>
       <c r="J13" s="22"/>
       <c r="K13" s="22">
@@ -2206,7 +2194,7 @@
         <v>10</v>
       </c>
       <c r="N13" s="35" t="s">
-        <v>169</v>
+        <v>162</v>
       </c>
       <c r="O13" s="25">
         <v>4.1700000000000001E-2</v>
@@ -2228,8 +2216,8 @@
       <c r="A14" s="7">
         <v>12</v>
       </c>
-      <c r="B14" s="41" t="s">
-        <v>164</v>
+      <c r="B14" s="57" t="s">
+        <v>157</v>
       </c>
       <c r="C14" s="8" t="s">
         <v>69</v>
@@ -2248,7 +2236,7 @@
       </c>
       <c r="H14" s="10"/>
       <c r="I14" s="10" t="s">
-        <v>187</v>
+        <v>180</v>
       </c>
       <c r="J14" s="9" t="s">
         <v>68</v>
@@ -2264,7 +2252,7 @@
         <v>5</v>
       </c>
       <c r="N14" s="35" t="s">
-        <v>169</v>
+        <v>162</v>
       </c>
       <c r="O14" s="11">
         <v>1.6999999999999999E-3</v>
@@ -2286,7 +2274,7 @@
       <c r="A15" s="7">
         <v>13</v>
       </c>
-      <c r="B15" s="46"/>
+      <c r="B15" s="62"/>
       <c r="C15" s="12" t="s">
         <v>75</v>
       </c>
@@ -2304,7 +2292,7 @@
       </c>
       <c r="H15" s="14"/>
       <c r="I15" s="14" t="s">
-        <v>188</v>
+        <v>181</v>
       </c>
       <c r="J15" s="13" t="s">
         <v>74</v>
@@ -2320,7 +2308,7 @@
         <v>25</v>
       </c>
       <c r="N15" s="35" t="s">
-        <v>169</v>
+        <v>162</v>
       </c>
       <c r="O15" s="15">
         <v>1.5E-3</v>
@@ -2333,7 +2321,7 @@
         <v>1.5E-3</v>
       </c>
       <c r="R15" s="11">
-        <f t="shared" ref="R15:R20" si="2">Q15*K15</f>
+        <f t="shared" ref="R15:R19" si="2">Q15*K15</f>
         <v>0.15</v>
       </c>
       <c r="S15" s="32"/>
@@ -2342,7 +2330,7 @@
       <c r="A16" s="7">
         <v>14</v>
       </c>
-      <c r="B16" s="46"/>
+      <c r="B16" s="62"/>
       <c r="C16" s="12" t="s">
         <v>79</v>
       </c>
@@ -2359,10 +2347,10 @@
         <v>83</v>
       </c>
       <c r="H16" s="14" t="s">
-        <v>189</v>
+        <v>182</v>
       </c>
       <c r="I16" s="14" t="s">
-        <v>190</v>
+        <v>183</v>
       </c>
       <c r="J16" s="13" t="s">
         <v>78</v>
@@ -2378,13 +2366,13 @@
         <v>5</v>
       </c>
       <c r="N16" s="35" t="s">
-        <v>169</v>
+        <v>162</v>
       </c>
       <c r="O16" s="15">
         <v>1.6000000000000001E-3</v>
       </c>
       <c r="P16" s="11">
-        <f t="shared" ref="P16:P20" si="3">O16*K16</f>
+        <f t="shared" ref="P16:P19" si="3">O16*K16</f>
         <v>0.16</v>
       </c>
       <c r="Q16" s="15">
@@ -2400,7 +2388,7 @@
       <c r="A17" s="7">
         <v>15</v>
       </c>
-      <c r="B17" s="46"/>
+      <c r="B17" s="62"/>
       <c r="C17" s="12" t="s">
         <v>85</v>
       </c>
@@ -2418,7 +2406,7 @@
       </c>
       <c r="H17" s="14"/>
       <c r="I17" s="14" t="s">
-        <v>191</v>
+        <v>184</v>
       </c>
       <c r="J17" s="13" t="s">
         <v>84</v>
@@ -2434,7 +2422,7 @@
         <v>10</v>
       </c>
       <c r="N17" s="35" t="s">
-        <v>169</v>
+        <v>162</v>
       </c>
       <c r="O17" s="15">
         <v>1.4E-3</v>
@@ -2456,7 +2444,7 @@
       <c r="A18" s="7">
         <v>16</v>
       </c>
-      <c r="B18" s="46"/>
+      <c r="B18" s="62"/>
       <c r="C18" s="12" t="s">
         <v>89</v>
       </c>
@@ -2474,7 +2462,7 @@
       </c>
       <c r="H18" s="14"/>
       <c r="I18" s="14" t="s">
-        <v>192</v>
+        <v>185</v>
       </c>
       <c r="J18" s="13" t="s">
         <v>88</v>
@@ -2490,7 +2478,7 @@
         <v>5</v>
       </c>
       <c r="N18" s="35" t="s">
-        <v>169</v>
+        <v>162</v>
       </c>
       <c r="O18" s="15">
         <v>2.3999999999999998E-3</v>
@@ -2512,28 +2500,28 @@
       <c r="A19" s="7">
         <v>17</v>
       </c>
-      <c r="B19" s="46"/>
+      <c r="B19" s="62"/>
       <c r="C19" s="12" t="s">
-        <v>93</v>
+        <v>193</v>
       </c>
       <c r="D19" s="13" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="E19" s="13" t="s">
         <v>71</v>
       </c>
-      <c r="F19" s="13" t="s">
-        <v>96</v>
+      <c r="F19" s="63" t="s">
+        <v>194</v>
       </c>
       <c r="G19" s="13" t="s">
-        <v>95</v>
+        <v>73</v>
       </c>
       <c r="H19" s="14"/>
       <c r="I19" s="14" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="J19" s="13" t="s">
-        <v>92</v>
+        <v>196</v>
       </c>
       <c r="K19" s="13">
         <v>50</v>
@@ -2546,363 +2534,359 @@
         <v>10</v>
       </c>
       <c r="N19" s="35" t="s">
-        <v>169</v>
+        <v>162</v>
       </c>
       <c r="O19" s="15">
-        <v>8.8000000000000005E-3</v>
+        <v>4.1000000000000003E-3</v>
       </c>
       <c r="P19" s="11">
         <f t="shared" si="3"/>
-        <v>0.44</v>
+        <v>0.20500000000000002</v>
       </c>
       <c r="Q19" s="15">
-        <v>8.8000000000000005E-3</v>
+        <v>4.1000000000000003E-3</v>
       </c>
       <c r="R19" s="11">
         <f t="shared" si="2"/>
-        <v>0.44</v>
+        <v>0.20500000000000002</v>
       </c>
       <c r="S19" s="32"/>
     </row>
     <row r="20" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="7">
-        <v>18</v>
-      </c>
-      <c r="B20" s="42"/>
-      <c r="C20" s="16" t="s">
-        <v>97</v>
-      </c>
-      <c r="D20" s="17" t="s">
-        <v>98</v>
-      </c>
-      <c r="E20" s="17" t="s">
-        <v>81</v>
-      </c>
-      <c r="F20" s="17" t="s">
-        <v>99</v>
-      </c>
-      <c r="G20" s="17" t="s">
-        <v>73</v>
-      </c>
-      <c r="H20" s="18"/>
-      <c r="I20" s="18" t="s">
-        <v>194</v>
-      </c>
-      <c r="J20" s="17" t="s">
-        <v>84</v>
-      </c>
-      <c r="K20" s="17">
-        <v>100</v>
-      </c>
-      <c r="L20" s="18">
-        <v>2</v>
-      </c>
-      <c r="M20" s="18">
+        <v>19</v>
+      </c>
+      <c r="B20" s="6" t="s">
+        <v>158</v>
+      </c>
+      <c r="C20" s="21" t="s">
+        <v>94</v>
+      </c>
+      <c r="D20" s="22" t="s">
+        <v>95</v>
+      </c>
+      <c r="E20" s="22" t="s">
+        <v>93</v>
+      </c>
+      <c r="F20" s="22" t="s">
+        <v>93</v>
+      </c>
+      <c r="G20" s="22" t="s">
+        <v>96</v>
+      </c>
+      <c r="H20" s="23"/>
+      <c r="I20" s="23" t="s">
+        <v>186</v>
+      </c>
+      <c r="J20" s="22"/>
+      <c r="K20" s="22">
+        <v>1</v>
+      </c>
+      <c r="L20" s="23">
+        <v>1</v>
+      </c>
+      <c r="M20" s="23">
         <f t="shared" si="0"/>
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="N20" s="35" t="s">
-        <v>169</v>
-      </c>
-      <c r="O20" s="19">
-        <v>1.1000000000000001E-3</v>
-      </c>
-      <c r="P20" s="11">
-        <f t="shared" si="3"/>
-        <v>0.11</v>
-      </c>
-      <c r="Q20" s="19">
-        <v>1.1000000000000001E-3</v>
-      </c>
-      <c r="R20" s="11">
-        <f t="shared" si="2"/>
-        <v>0.11</v>
-      </c>
-      <c r="S20" s="33"/>
+        <v>162</v>
+      </c>
+      <c r="O20" s="25">
+        <v>0.47610000000000002</v>
+      </c>
+      <c r="P20" s="25">
+        <f t="shared" ref="P20:P31" si="4">O20*L20</f>
+        <v>0.47610000000000002</v>
+      </c>
+      <c r="Q20" s="25">
+        <v>0.47610000000000002</v>
+      </c>
+      <c r="R20" s="25">
+        <f t="shared" si="1"/>
+        <v>2.3805000000000001</v>
+      </c>
+      <c r="S20" s="34"/>
     </row>
     <row r="21" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="7">
-        <v>19</v>
-      </c>
-      <c r="B21" s="6" t="s">
-        <v>165</v>
-      </c>
-      <c r="C21" s="21" t="s">
-        <v>101</v>
-      </c>
-      <c r="D21" s="22" t="s">
-        <v>102</v>
-      </c>
-      <c r="E21" s="22" t="s">
-        <v>100</v>
-      </c>
-      <c r="F21" s="22" t="s">
-        <v>100</v>
-      </c>
-      <c r="G21" s="22" t="s">
-        <v>103</v>
-      </c>
-      <c r="H21" s="23"/>
-      <c r="I21" s="23" t="s">
-        <v>195</v>
-      </c>
-      <c r="J21" s="22"/>
-      <c r="K21" s="22">
+        <v>20</v>
+      </c>
+      <c r="B21" s="57" t="s">
+        <v>159</v>
+      </c>
+      <c r="C21" s="8" t="s">
+        <v>131</v>
+      </c>
+      <c r="D21" s="9" t="s">
+        <v>132</v>
+      </c>
+      <c r="E21" s="9" t="s">
+        <v>133</v>
+      </c>
+      <c r="F21" s="9" t="s">
+        <v>133</v>
+      </c>
+      <c r="G21" s="9" t="s">
+        <v>134</v>
+      </c>
+      <c r="H21" s="10"/>
+      <c r="I21" s="10" t="s">
+        <v>187</v>
+      </c>
+      <c r="J21" s="9" t="s">
+        <v>130</v>
+      </c>
+      <c r="K21" s="9">
         <v>1</v>
       </c>
-      <c r="L21" s="23">
+      <c r="L21" s="10">
         <v>1</v>
       </c>
-      <c r="M21" s="23">
+      <c r="M21" s="10">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
       <c r="N21" s="35" t="s">
-        <v>169</v>
-      </c>
-      <c r="O21" s="25">
-        <v>0.47610000000000002</v>
-      </c>
-      <c r="P21" s="25">
-        <f t="shared" ref="P21:P32" si="4">O21*L21</f>
-        <v>0.47610000000000002</v>
-      </c>
-      <c r="Q21" s="25">
-        <v>0.47610000000000002</v>
-      </c>
-      <c r="R21" s="25">
+        <v>162</v>
+      </c>
+      <c r="O21" s="11">
+        <v>0.3634</v>
+      </c>
+      <c r="P21" s="11">
+        <f t="shared" si="4"/>
+        <v>0.3634</v>
+      </c>
+      <c r="Q21" s="11">
+        <v>0.3634</v>
+      </c>
+      <c r="R21" s="11">
         <f t="shared" si="1"/>
-        <v>2.3805000000000001</v>
-      </c>
-      <c r="S21" s="34"/>
+        <v>1.8169999999999999</v>
+      </c>
+      <c r="S21" s="31"/>
     </row>
     <row r="22" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="7">
-        <v>20</v>
-      </c>
-      <c r="B22" s="41" t="s">
-        <v>166</v>
-      </c>
-      <c r="C22" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="B22" s="58"/>
+      <c r="C22" s="16" t="s">
+        <v>136</v>
+      </c>
+      <c r="D22" s="17" t="s">
+        <v>137</v>
+      </c>
+      <c r="E22" s="17" t="s">
+        <v>135</v>
+      </c>
+      <c r="F22" s="17" t="s">
+        <v>135</v>
+      </c>
+      <c r="G22" s="17" t="s">
         <v>138</v>
       </c>
-      <c r="D22" s="9" t="s">
-        <v>139</v>
-      </c>
-      <c r="E22" s="9" t="s">
-        <v>140</v>
-      </c>
-      <c r="F22" s="9" t="s">
-        <v>140</v>
-      </c>
-      <c r="G22" s="9" t="s">
-        <v>141</v>
-      </c>
-      <c r="H22" s="10"/>
-      <c r="I22" s="10" t="s">
-        <v>196</v>
-      </c>
-      <c r="J22" s="9" t="s">
-        <v>137</v>
-      </c>
-      <c r="K22" s="9">
+      <c r="H22" s="18"/>
+      <c r="I22" s="18"/>
+      <c r="J22" s="17"/>
+      <c r="K22" s="17">
         <v>1</v>
       </c>
-      <c r="L22" s="10">
+      <c r="L22" s="18">
         <v>1</v>
       </c>
-      <c r="M22" s="10">
+      <c r="M22" s="18">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
       <c r="N22" s="35" t="s">
-        <v>169</v>
-      </c>
-      <c r="O22" s="11">
-        <v>0.3634</v>
-      </c>
-      <c r="P22" s="11">
+        <v>188</v>
+      </c>
+      <c r="O22" s="19">
+        <v>0.71889999999999998</v>
+      </c>
+      <c r="P22" s="19">
         <f t="shared" si="4"/>
-        <v>0.3634</v>
-      </c>
-      <c r="Q22" s="11">
-        <v>0.3634</v>
-      </c>
-      <c r="R22" s="11">
+        <v>0.71889999999999998</v>
+      </c>
+      <c r="Q22" s="19">
+        <v>0.71889999999999998</v>
+      </c>
+      <c r="R22" s="19">
         <f t="shared" si="1"/>
-        <v>1.8169999999999999</v>
-      </c>
-      <c r="S22" s="31"/>
+        <v>3.5945</v>
+      </c>
+      <c r="S22" s="33"/>
     </row>
     <row r="23" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="7">
-        <v>21</v>
-      </c>
-      <c r="B23" s="42"/>
-      <c r="C23" s="16" t="s">
-        <v>143</v>
-      </c>
-      <c r="D23" s="17" t="s">
-        <v>144</v>
-      </c>
-      <c r="E23" s="17" t="s">
-        <v>142</v>
-      </c>
-      <c r="F23" s="17" t="s">
-        <v>142</v>
-      </c>
-      <c r="G23" s="17" t="s">
-        <v>145</v>
-      </c>
-      <c r="H23" s="18"/>
-      <c r="I23" s="18"/>
-      <c r="J23" s="17"/>
-      <c r="K23" s="17">
+        <v>22</v>
+      </c>
+      <c r="B23" s="57" t="s">
+        <v>160</v>
+      </c>
+      <c r="C23" s="39" t="s">
+        <v>98</v>
+      </c>
+      <c r="D23" s="40" t="s">
+        <v>99</v>
+      </c>
+      <c r="E23" s="40" t="s">
+        <v>100</v>
+      </c>
+      <c r="F23" s="40" t="s">
+        <v>97</v>
+      </c>
+      <c r="G23" s="40" t="s">
+        <v>101</v>
+      </c>
+      <c r="H23" s="41"/>
+      <c r="I23" s="41"/>
+      <c r="J23" s="40"/>
+      <c r="K23" s="40"/>
+      <c r="L23" s="41">
         <v>1</v>
       </c>
-      <c r="L23" s="18">
-        <v>1</v>
-      </c>
-      <c r="M23" s="18">
+      <c r="M23" s="41">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="N23" s="35" t="s">
-        <v>197</v>
-      </c>
-      <c r="O23" s="19">
-        <v>0.71889999999999998</v>
-      </c>
-      <c r="P23" s="19">
+      <c r="N23" s="42" t="s">
+        <v>162</v>
+      </c>
+      <c r="O23" s="50"/>
+      <c r="P23" s="44">
         <f t="shared" si="4"/>
-        <v>0.71889999999999998</v>
-      </c>
-      <c r="Q23" s="19">
-        <v>0.71889999999999998</v>
-      </c>
-      <c r="R23" s="19">
+        <v>0</v>
+      </c>
+      <c r="Q23" s="50"/>
+      <c r="R23" s="44">
         <f t="shared" si="1"/>
-        <v>3.5945</v>
-      </c>
-      <c r="S23" s="33"/>
+        <v>0</v>
+      </c>
+      <c r="S23" s="49" t="s">
+        <v>192</v>
+      </c>
     </row>
     <row r="24" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="7">
-        <v>22</v>
-      </c>
-      <c r="B24" s="41" t="s">
-        <v>167</v>
-      </c>
-      <c r="C24" s="47" t="s">
+        <v>23</v>
+      </c>
+      <c r="B24" s="62"/>
+      <c r="C24" s="51" t="s">
+        <v>103</v>
+      </c>
+      <c r="D24" s="52" t="s">
+        <v>104</v>
+      </c>
+      <c r="E24" s="52" t="s">
         <v>105</v>
       </c>
-      <c r="D24" s="48" t="s">
+      <c r="F24" s="52" t="s">
+        <v>102</v>
+      </c>
+      <c r="G24" s="52" t="s">
         <v>106</v>
       </c>
-      <c r="E24" s="48" t="s">
-        <v>107</v>
-      </c>
-      <c r="F24" s="48" t="s">
-        <v>104</v>
-      </c>
-      <c r="G24" s="48" t="s">
-        <v>108</v>
-      </c>
-      <c r="H24" s="49"/>
-      <c r="I24" s="49"/>
-      <c r="J24" s="48"/>
-      <c r="K24" s="48"/>
-      <c r="L24" s="49">
+      <c r="H24" s="53"/>
+      <c r="I24" s="53"/>
+      <c r="J24" s="52"/>
+      <c r="K24" s="52"/>
+      <c r="L24" s="53">
         <v>1</v>
       </c>
-      <c r="M24" s="49">
+      <c r="M24" s="53">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="N24" s="50" t="s">
-        <v>169</v>
-      </c>
-      <c r="O24" s="58"/>
-      <c r="P24" s="52">
+      <c r="N24" s="42" t="s">
+        <v>162</v>
+      </c>
+      <c r="O24" s="54"/>
+      <c r="P24" s="54">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="Q24" s="58"/>
-      <c r="R24" s="52">
+      <c r="Q24" s="54"/>
+      <c r="R24" s="54">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="S24" s="57" t="s">
-        <v>201</v>
+      <c r="S24" s="49" t="s">
+        <v>192</v>
       </c>
     </row>
     <row r="25" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="7">
-        <v>23</v>
-      </c>
-      <c r="B25" s="46"/>
-      <c r="C25" s="59" t="s">
+        <v>24</v>
+      </c>
+      <c r="B25" s="62"/>
+      <c r="C25" s="12" t="s">
+        <v>108</v>
+      </c>
+      <c r="D25" s="13" t="s">
+        <v>109</v>
+      </c>
+      <c r="E25" s="13" t="s">
         <v>110</v>
       </c>
-      <c r="D25" s="60" t="s">
+      <c r="F25" s="13" t="s">
+        <v>107</v>
+      </c>
+      <c r="G25" s="13" t="s">
         <v>111</v>
       </c>
-      <c r="E25" s="60" t="s">
-        <v>112</v>
-      </c>
-      <c r="F25" s="60" t="s">
-        <v>109</v>
-      </c>
-      <c r="G25" s="60" t="s">
-        <v>113</v>
-      </c>
-      <c r="H25" s="61"/>
-      <c r="I25" s="61"/>
-      <c r="J25" s="60"/>
-      <c r="K25" s="60"/>
-      <c r="L25" s="61">
+      <c r="H25" s="14"/>
+      <c r="I25" s="14"/>
+      <c r="J25" s="13"/>
+      <c r="K25" s="13">
         <v>1</v>
       </c>
-      <c r="M25" s="61">
+      <c r="L25" s="14">
+        <v>1</v>
+      </c>
+      <c r="M25" s="14">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="N25" s="50" t="s">
-        <v>169</v>
-      </c>
-      <c r="O25" s="62"/>
-      <c r="P25" s="62">
+      <c r="N25" s="35" t="s">
+        <v>191</v>
+      </c>
+      <c r="O25" s="26">
+        <v>7.6</v>
+      </c>
+      <c r="P25" s="15">
         <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="Q25" s="62"/>
-      <c r="R25" s="62">
+        <v>7.6</v>
+      </c>
+      <c r="Q25" s="26">
+        <v>7.6</v>
+      </c>
+      <c r="R25" s="15">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="S25" s="57" t="s">
-        <v>201</v>
-      </c>
+        <v>38</v>
+      </c>
+      <c r="S25" s="32"/>
     </row>
     <row r="26" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="7">
-        <v>24</v>
-      </c>
-      <c r="B26" s="46"/>
+        <v>25</v>
+      </c>
+      <c r="B26" s="62"/>
       <c r="C26" s="12" t="s">
+        <v>113</v>
+      </c>
+      <c r="D26" s="13" t="s">
+        <v>114</v>
+      </c>
+      <c r="E26" s="13" t="s">
         <v>115</v>
       </c>
-      <c r="D26" s="13" t="s">
+      <c r="F26" s="13" t="s">
+        <v>112</v>
+      </c>
+      <c r="G26" s="13" t="s">
         <v>116</v>
-      </c>
-      <c r="E26" s="13" t="s">
-        <v>117</v>
-      </c>
-      <c r="F26" s="13" t="s">
-        <v>114</v>
-      </c>
-      <c r="G26" s="13" t="s">
-        <v>118</v>
       </c>
       <c r="H26" s="14"/>
       <c r="I26" s="14"/>
@@ -2918,46 +2902,48 @@
         <v>5</v>
       </c>
       <c r="N26" s="35" t="s">
-        <v>200</v>
-      </c>
-      <c r="O26" s="26">
-        <v>7.6</v>
+        <v>165</v>
+      </c>
+      <c r="O26" s="27">
+        <v>11</v>
       </c>
       <c r="P26" s="15">
-        <f t="shared" si="4"/>
-        <v>7.6</v>
-      </c>
-      <c r="Q26" s="26">
-        <v>7.6</v>
+        <f>O26*L26</f>
+        <v>11</v>
+      </c>
+      <c r="Q26" s="27">
+        <v>11</v>
       </c>
       <c r="R26" s="15">
-        <f t="shared" si="1"/>
-        <v>38</v>
+        <f>Q26*M26</f>
+        <v>55</v>
       </c>
       <c r="S26" s="32"/>
     </row>
     <row r="27" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="7">
-        <v>25</v>
-      </c>
-      <c r="B27" s="46"/>
+        <v>26</v>
+      </c>
+      <c r="B27" s="62"/>
       <c r="C27" s="12" t="s">
+        <v>118</v>
+      </c>
+      <c r="D27" s="13" t="s">
+        <v>119</v>
+      </c>
+      <c r="E27" s="13" t="s">
         <v>120</v>
       </c>
-      <c r="D27" s="13" t="s">
-        <v>121</v>
-      </c>
-      <c r="E27" s="13" t="s">
-        <v>122</v>
-      </c>
       <c r="F27" s="13" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="G27" s="13" t="s">
-        <v>123</v>
+        <v>106</v>
       </c>
       <c r="H27" s="14"/>
-      <c r="I27" s="14"/>
+      <c r="I27" s="14" t="s">
+        <v>189</v>
+      </c>
       <c r="J27" s="13"/>
       <c r="K27" s="13">
         <v>1</v>
@@ -2970,48 +2956,46 @@
         <v>5</v>
       </c>
       <c r="N27" s="35" t="s">
-        <v>172</v>
-      </c>
-      <c r="O27" s="27">
-        <v>11</v>
+        <v>162</v>
+      </c>
+      <c r="O27" s="15">
+        <v>0.18190000000000001</v>
       </c>
       <c r="P27" s="15">
-        <f>O27*L27</f>
-        <v>11</v>
-      </c>
-      <c r="Q27" s="27">
-        <v>11</v>
+        <f t="shared" si="4"/>
+        <v>0.18190000000000001</v>
+      </c>
+      <c r="Q27" s="15">
+        <v>0.18190000000000001</v>
       </c>
       <c r="R27" s="15">
-        <f>Q27*M27</f>
-        <v>55</v>
+        <f t="shared" si="1"/>
+        <v>0.90949999999999998</v>
       </c>
       <c r="S27" s="32"/>
     </row>
     <row r="28" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="7">
-        <v>26</v>
-      </c>
-      <c r="B28" s="46"/>
+        <v>27</v>
+      </c>
+      <c r="B28" s="62"/>
       <c r="C28" s="12" t="s">
+        <v>122</v>
+      </c>
+      <c r="D28" s="13" t="s">
+        <v>123</v>
+      </c>
+      <c r="E28" s="13" t="s">
+        <v>124</v>
+      </c>
+      <c r="F28" s="13" t="s">
+        <v>121</v>
+      </c>
+      <c r="G28" s="13" t="s">
         <v>125</v>
       </c>
-      <c r="D28" s="13" t="s">
-        <v>126</v>
-      </c>
-      <c r="E28" s="13" t="s">
-        <v>127</v>
-      </c>
-      <c r="F28" s="13" t="s">
-        <v>124</v>
-      </c>
-      <c r="G28" s="13" t="s">
-        <v>113</v>
-      </c>
       <c r="H28" s="14"/>
-      <c r="I28" s="14" t="s">
-        <v>198</v>
-      </c>
+      <c r="I28" s="14"/>
       <c r="J28" s="13"/>
       <c r="K28" s="13">
         <v>1</v>
@@ -3024,268 +3008,230 @@
         <v>5</v>
       </c>
       <c r="N28" s="35" t="s">
-        <v>169</v>
+        <v>191</v>
       </c>
       <c r="O28" s="15">
-        <v>0.18190000000000001</v>
+        <v>0.85</v>
       </c>
       <c r="P28" s="15">
         <f t="shared" si="4"/>
-        <v>0.18190000000000001</v>
+        <v>0.85</v>
       </c>
       <c r="Q28" s="15">
-        <v>0.18190000000000001</v>
+        <v>0.85</v>
       </c>
       <c r="R28" s="15">
         <f t="shared" si="1"/>
-        <v>0.90949999999999998</v>
+        <v>4.25</v>
       </c>
       <c r="S28" s="32"/>
     </row>
     <row r="29" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="7">
-        <v>27</v>
-      </c>
-      <c r="B29" s="46"/>
-      <c r="C29" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="B29" s="58"/>
+      <c r="C29" s="16" t="s">
+        <v>127</v>
+      </c>
+      <c r="D29" s="17" t="s">
+        <v>128</v>
+      </c>
+      <c r="E29" s="17" t="s">
         <v>129</v>
       </c>
-      <c r="D29" s="13" t="s">
-        <v>130</v>
-      </c>
-      <c r="E29" s="13" t="s">
-        <v>131</v>
-      </c>
-      <c r="F29" s="13" t="s">
-        <v>128</v>
-      </c>
-      <c r="G29" s="13" t="s">
-        <v>132</v>
-      </c>
-      <c r="H29" s="14"/>
-      <c r="I29" s="14"/>
-      <c r="J29" s="13"/>
-      <c r="K29" s="13">
+      <c r="F29" s="17" t="s">
+        <v>126</v>
+      </c>
+      <c r="G29" s="17" t="s">
+        <v>44</v>
+      </c>
+      <c r="H29" s="18"/>
+      <c r="I29" s="18"/>
+      <c r="J29" s="17"/>
+      <c r="K29" s="17">
         <v>1</v>
       </c>
-      <c r="L29" s="14">
+      <c r="L29" s="18">
         <v>1</v>
       </c>
-      <c r="M29" s="14">
+      <c r="M29" s="18">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
       <c r="N29" s="35" t="s">
-        <v>200</v>
-      </c>
-      <c r="O29" s="15">
-        <v>0.85</v>
-      </c>
-      <c r="P29" s="15">
+        <v>190</v>
+      </c>
+      <c r="O29" s="19">
+        <v>0.19600000000000001</v>
+      </c>
+      <c r="P29" s="19">
         <f t="shared" si="4"/>
-        <v>0.85</v>
-      </c>
-      <c r="Q29" s="15">
-        <v>0.85</v>
-      </c>
-      <c r="R29" s="15">
+        <v>0.19600000000000001</v>
+      </c>
+      <c r="Q29" s="19">
+        <v>0.19600000000000001</v>
+      </c>
+      <c r="R29" s="19">
         <f t="shared" si="1"/>
-        <v>4.25</v>
-      </c>
-      <c r="S29" s="32"/>
+        <v>0.98</v>
+      </c>
+      <c r="S29" s="33"/>
     </row>
     <row r="30" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="7">
-        <v>28</v>
-      </c>
-      <c r="B30" s="42"/>
-      <c r="C30" s="16" t="s">
-        <v>134</v>
-      </c>
-      <c r="D30" s="17" t="s">
-        <v>135</v>
-      </c>
-      <c r="E30" s="17" t="s">
-        <v>136</v>
-      </c>
-      <c r="F30" s="17" t="s">
-        <v>133</v>
-      </c>
-      <c r="G30" s="17" t="s">
-        <v>44</v>
-      </c>
-      <c r="H30" s="18"/>
-      <c r="I30" s="18"/>
-      <c r="J30" s="17"/>
-      <c r="K30" s="17">
+        <v>29</v>
+      </c>
+      <c r="B30" s="57" t="s">
+        <v>161</v>
+      </c>
+      <c r="C30" s="39" t="s">
+        <v>46</v>
+      </c>
+      <c r="D30" s="40" t="s">
+        <v>47</v>
+      </c>
+      <c r="E30" s="40" t="s">
+        <v>45</v>
+      </c>
+      <c r="F30" s="40" t="s">
+        <v>45</v>
+      </c>
+      <c r="G30" s="40" t="s">
+        <v>48</v>
+      </c>
+      <c r="H30" s="41"/>
+      <c r="I30" s="41"/>
+      <c r="J30" s="40"/>
+      <c r="K30" s="40"/>
+      <c r="L30" s="41">
         <v>1</v>
       </c>
-      <c r="L30" s="18">
-        <v>1</v>
-      </c>
-      <c r="M30" s="18">
+      <c r="M30" s="41">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="N30" s="35" t="s">
-        <v>199</v>
-      </c>
-      <c r="O30" s="19">
-        <v>0.19600000000000001</v>
-      </c>
-      <c r="P30" s="19">
+      <c r="N30" s="42" t="s">
+        <v>162</v>
+      </c>
+      <c r="O30" s="43"/>
+      <c r="P30" s="44">
         <f t="shared" si="4"/>
-        <v>0.19600000000000001</v>
-      </c>
-      <c r="Q30" s="19">
-        <v>0.19600000000000001</v>
-      </c>
-      <c r="R30" s="19">
+        <v>0</v>
+      </c>
+      <c r="Q30" s="43"/>
+      <c r="R30" s="44">
         <f t="shared" si="1"/>
-        <v>0.98</v>
-      </c>
-      <c r="S30" s="33"/>
+        <v>0</v>
+      </c>
+      <c r="S30" s="49" t="s">
+        <v>192</v>
+      </c>
     </row>
     <row r="31" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="7">
-        <v>29</v>
-      </c>
-      <c r="B31" s="41" t="s">
-        <v>168</v>
-      </c>
-      <c r="C31" s="47" t="s">
-        <v>46</v>
-      </c>
-      <c r="D31" s="48" t="s">
-        <v>47</v>
-      </c>
-      <c r="E31" s="48" t="s">
-        <v>45</v>
-      </c>
-      <c r="F31" s="48" t="s">
-        <v>45</v>
-      </c>
-      <c r="G31" s="48" t="s">
-        <v>48</v>
-      </c>
-      <c r="H31" s="49"/>
-      <c r="I31" s="49"/>
-      <c r="J31" s="48"/>
-      <c r="K31" s="48"/>
-      <c r="L31" s="49">
+        <v>30</v>
+      </c>
+      <c r="B31" s="58"/>
+      <c r="C31" s="45" t="s">
+        <v>60</v>
+      </c>
+      <c r="D31" s="46" t="s">
+        <v>61</v>
+      </c>
+      <c r="E31" s="46" t="s">
+        <v>59</v>
+      </c>
+      <c r="F31" s="46" t="s">
+        <v>59</v>
+      </c>
+      <c r="G31" s="46" t="s">
+        <v>62</v>
+      </c>
+      <c r="H31" s="47"/>
+      <c r="I31" s="47"/>
+      <c r="J31" s="46"/>
+      <c r="K31" s="46"/>
+      <c r="L31" s="47">
         <v>1</v>
       </c>
-      <c r="M31" s="49">
+      <c r="M31" s="47">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="N31" s="50" t="s">
-        <v>169</v>
-      </c>
-      <c r="O31" s="51"/>
-      <c r="P31" s="52">
+      <c r="N31" s="42" t="s">
+        <v>162</v>
+      </c>
+      <c r="O31" s="47"/>
+      <c r="P31" s="48">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="Q31" s="51"/>
-      <c r="R31" s="52">
+      <c r="Q31" s="48"/>
+      <c r="R31" s="48">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="S31" s="57" t="s">
-        <v>201</v>
+      <c r="S31" s="49" t="s">
+        <v>192</v>
       </c>
     </row>
-    <row r="32" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="7">
-        <v>30</v>
-      </c>
-      <c r="B32" s="42"/>
-      <c r="C32" s="53" t="s">
-        <v>60</v>
-      </c>
-      <c r="D32" s="54" t="s">
-        <v>61</v>
-      </c>
-      <c r="E32" s="54" t="s">
-        <v>59</v>
-      </c>
-      <c r="F32" s="54" t="s">
-        <v>59</v>
-      </c>
-      <c r="G32" s="54" t="s">
-        <v>62</v>
-      </c>
-      <c r="H32" s="55"/>
-      <c r="I32" s="55"/>
-      <c r="J32" s="54"/>
-      <c r="K32" s="54"/>
-      <c r="L32" s="55">
-        <v>1</v>
-      </c>
-      <c r="M32" s="55">
-        <f t="shared" si="0"/>
-        <v>5</v>
-      </c>
-      <c r="N32" s="50" t="s">
-        <v>169</v>
-      </c>
+    <row r="32" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="L32" s="55" t="s">
+        <v>163</v>
+      </c>
+      <c r="M32" s="55"/>
+      <c r="N32" s="55"/>
       <c r="O32" s="55"/>
-      <c r="P32" s="56">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="Q32" s="56"/>
-      <c r="R32" s="56">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="S32" s="57" t="s">
-        <v>201</v>
+      <c r="R32" s="3">
+        <f>SUM(R3:R31)</f>
+        <v>117.0955</v>
       </c>
     </row>
-    <row r="33" spans="12:18" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="L33" s="39" t="s">
-        <v>170</v>
-      </c>
-      <c r="M33" s="39"/>
-      <c r="N33" s="39"/>
-      <c r="O33" s="39"/>
-      <c r="R33" s="3">
-        <f>SUM(R3:R32)</f>
-        <v>117.4405</v>
-      </c>
-    </row>
-    <row r="34" spans="12:18" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="L34" s="40" t="s">
-        <v>171</v>
-      </c>
-      <c r="M34" s="40"/>
-      <c r="N34" s="40"/>
-      <c r="O34" s="40"/>
-      <c r="P34" s="2">
-        <f>SUM(P3:P32)</f>
-        <v>30.840300000000003</v>
-      </c>
-      <c r="R34" s="4">
-        <f>R33/5</f>
-        <v>23.488099999999999</v>
+    <row r="33" spans="12:18" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="L33" s="56" t="s">
+        <v>164</v>
+      </c>
+      <c r="M33" s="56"/>
+      <c r="N33" s="56"/>
+      <c r="O33" s="56"/>
+      <c r="P33" s="2">
+        <f>SUM(P3:P31)</f>
+        <v>30.495300000000004</v>
+      </c>
+      <c r="R33" s="4">
+        <f>R32/5</f>
+        <v>23.4191</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="9">
+    <mergeCell ref="L32:O32"/>
     <mergeCell ref="L33:O33"/>
-    <mergeCell ref="L34:O34"/>
-    <mergeCell ref="B31:B32"/>
+    <mergeCell ref="B30:B31"/>
     <mergeCell ref="A1:S1"/>
     <mergeCell ref="B3:B8"/>
     <mergeCell ref="B9:B11"/>
-    <mergeCell ref="B14:B20"/>
-    <mergeCell ref="B22:B23"/>
-    <mergeCell ref="B24:B30"/>
+    <mergeCell ref="B14:B19"/>
+    <mergeCell ref="B21:B22"/>
+    <mergeCell ref="B23:B29"/>
   </mergeCells>
-  <conditionalFormatting sqref="L3:M32">
-    <cfRule type="colorScale" priority="6">
+  <conditionalFormatting sqref="P33:R33">
+    <cfRule type="dataBar" priority="3">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FF63C384"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{70EE1023-228D-423C-ADF5-29102BB53C0F}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L3:M31">
+    <cfRule type="colorScale" priority="7">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -3296,8 +3242,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P3:P32">
-    <cfRule type="dataBar" priority="5">
+  <conditionalFormatting sqref="P3:P31">
+    <cfRule type="dataBar" priority="9">
       <dataBar>
         <cfvo type="min"/>
         <cfvo type="max"/>
@@ -3310,8 +3256,8 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="R3:R32">
-    <cfRule type="dataBar" priority="4">
+  <conditionalFormatting sqref="R3:R31">
+    <cfRule type="dataBar" priority="11">
       <dataBar>
         <cfvo type="min"/>
         <cfvo type="max"/>
@@ -3320,20 +3266,6 @@
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
           <x14:id>{BC439CAB-0450-4930-B07F-0CD52FB2A12C}</x14:id>
-        </ext>
-      </extLst>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="P34:R34">
-    <cfRule type="dataBar" priority="3">
-      <dataBar>
-        <cfvo type="min"/>
-        <cfvo type="max"/>
-        <color rgb="FF63C384"/>
-      </dataBar>
-      <extLst>
-        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{70EE1023-228D-423C-ADF5-29102BB53C0F}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -3356,22 +3288,34 @@
     <hyperlink ref="N17" r:id="rId15" xr:uid="{BB3E0003-37A7-4A33-A7C7-BD7D81F75052}"/>
     <hyperlink ref="N18" r:id="rId16" xr:uid="{227291DF-41F8-4C10-AD55-6E82F7F2BDB8}"/>
     <hyperlink ref="N19" r:id="rId17" xr:uid="{78C7968A-0AD4-4927-B140-C8A8581C1A99}"/>
-    <hyperlink ref="N20" r:id="rId18" xr:uid="{F56CB4D3-A70E-49F6-AF0A-6498CD88639A}"/>
-    <hyperlink ref="N21" r:id="rId19" xr:uid="{6C8B6C89-82E9-4D35-BF15-26CF6D16AC05}"/>
-    <hyperlink ref="N22" r:id="rId20" xr:uid="{B3AA4E3D-0A25-4066-8A80-3F4EE2945B80}"/>
-    <hyperlink ref="N23" r:id="rId21" xr:uid="{3B123718-832D-454C-BF98-3C3488E403CB}"/>
-    <hyperlink ref="N28" r:id="rId22" xr:uid="{46AFA74C-C909-43C2-9FFC-8DA5DE966597}"/>
-    <hyperlink ref="N30" r:id="rId23" xr:uid="{07803BFD-F478-4F72-B06A-95A70758BAE3}"/>
-    <hyperlink ref="N29" r:id="rId24" xr:uid="{0789898D-0603-42C1-9FAE-7FBD24806F7D}"/>
-    <hyperlink ref="N27" r:id="rId25" xr:uid="{4CF7CCB5-DF91-46B6-9D91-E81CD0728CA9}"/>
-    <hyperlink ref="N26" r:id="rId26" xr:uid="{7F769DA7-F115-4FCB-8955-2D8B2FD08D98}"/>
+    <hyperlink ref="N20" r:id="rId18" xr:uid="{6C8B6C89-82E9-4D35-BF15-26CF6D16AC05}"/>
+    <hyperlink ref="N21" r:id="rId19" xr:uid="{B3AA4E3D-0A25-4066-8A80-3F4EE2945B80}"/>
+    <hyperlink ref="N22" r:id="rId20" xr:uid="{3B123718-832D-454C-BF98-3C3488E403CB}"/>
+    <hyperlink ref="N27" r:id="rId21" xr:uid="{46AFA74C-C909-43C2-9FFC-8DA5DE966597}"/>
+    <hyperlink ref="N29" r:id="rId22" xr:uid="{07803BFD-F478-4F72-B06A-95A70758BAE3}"/>
+    <hyperlink ref="N28" r:id="rId23" xr:uid="{0789898D-0603-42C1-9FAE-7FBD24806F7D}"/>
+    <hyperlink ref="N26" r:id="rId24" xr:uid="{4CF7CCB5-DF91-46B6-9D91-E81CD0728CA9}"/>
+    <hyperlink ref="N25" r:id="rId25" xr:uid="{7F769DA7-F115-4FCB-8955-2D8B2FD08D98}"/>
   </hyperlinks>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.30555555555555558" right="0.30555555555555558" top="0.30555555555555558" bottom="0.30555555555555558" header="0" footer="0"/>
-  <pageSetup scale="39" orientation="landscape" blackAndWhite="1" r:id="rId27"/>
+  <pageSetup scale="39" orientation="landscape" blackAndWhite="1" r:id="rId26"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="dataBar" id="{70EE1023-228D-423C-ADF5-29102BB53C0F}">
+            <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
+              <x14:cfvo type="autoMin"/>
+              <x14:cfvo type="autoMax"/>
+              <x14:borderColor rgb="FF63C384"/>
+              <x14:negativeFillColor rgb="FFFF0000"/>
+              <x14:negativeBorderColor rgb="FFFF0000"/>
+              <x14:axisColor rgb="FF000000"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <xm:sqref>P33:R33</xm:sqref>
+        </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
           <x14:cfRule type="dataBar" id="{31993F18-4C5F-4176-9D23-BFACE9C28768}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
@@ -3383,7 +3327,7 @@
               <x14:axisColor rgb="FF000000"/>
             </x14:dataBar>
           </x14:cfRule>
-          <xm:sqref>P3:P32</xm:sqref>
+          <xm:sqref>P3:P31</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
           <x14:cfRule type="dataBar" id="{BC439CAB-0450-4930-B07F-0CD52FB2A12C}">
@@ -3396,20 +3340,7 @@
               <x14:axisColor rgb="FF000000"/>
             </x14:dataBar>
           </x14:cfRule>
-          <xm:sqref>R3:R32</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{70EE1023-228D-423C-ADF5-29102BB53C0F}">
-            <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
-              <x14:cfvo type="autoMin"/>
-              <x14:cfvo type="autoMax"/>
-              <x14:borderColor rgb="FF63C384"/>
-              <x14:negativeFillColor rgb="FFFF0000"/>
-              <x14:negativeBorderColor rgb="FFFF0000"/>
-              <x14:axisColor rgb="FF000000"/>
-            </x14:dataBar>
-          </x14:cfRule>
-          <xm:sqref>P34:R34</xm:sqref>
+          <xm:sqref>R3:R31</xm:sqref>
         </x14:conditionalFormatting>
       </x14:conditionalFormattings>
     </ext>

</xml_diff>

<commit_message>
Alternate added for ESD diodes and X2 #95
</commit_message>
<xml_diff>
--- a/Deliverables/SM_Bottom Board/_BOM/SM_Bottom_Board_LCSC.xlsx
+++ b/Deliverables/SM_Bottom Board/_BOM/SM_Bottom_Board_LCSC.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\ColeBenson-SmartMotors\Deliverables\SM_Bottom Board\_BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark\ColeBenson-SmartMotors\Deliverables\SM_Bottom Board\_BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17D6AA03-4E0B-4BBE-9E77-171D15DF4C35}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C15AA912-DC7A-467D-8937-B48D35FCAE26}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SM_Bottom_Board" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,7 @@
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">SM_Bottom_Board!#REF!</definedName>
   </definedNames>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="338" uniqueCount="230">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="339" uniqueCount="234">
   <si>
     <t>Bill of Material (BOM) for Cole Benson</t>
   </si>
@@ -725,6 +725,18 @@
   </si>
   <si>
     <t>C845116</t>
+  </si>
+  <si>
+    <t>ESD5451N-TP</t>
+  </si>
+  <si>
+    <t>C2830311</t>
+  </si>
+  <si>
+    <t>FC31M2-32.768-N09LLDT</t>
+  </si>
+  <si>
+    <t>C2848222</t>
   </si>
 </sst>
 </file>
@@ -734,9 +746,9 @@
   <numFmts count="5">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.0000"/>
     <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.0000_);[Red]\(&quot;$&quot;#,##0.0000\)"/>
-    <numFmt numFmtId="168" formatCode="_-[$$-409]* #,##0.00_ ;_-[$$-409]* \-#,##0.00\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
-    <numFmt numFmtId="169" formatCode="&quot;$&quot;#,##0.000"/>
-    <numFmt numFmtId="170" formatCode="&quot;$&quot;#,##0.00"/>
+    <numFmt numFmtId="166" formatCode="_-[$$-409]* #,##0.00_ ;_-[$$-409]* \-#,##0.00\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
+    <numFmt numFmtId="167" formatCode="&quot;$&quot;#,##0.000"/>
+    <numFmt numFmtId="168" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
   <fonts count="24">
     <font>
@@ -1337,20 +1349,14 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="169" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="170" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="167" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1538,12 +1544,6 @@
     <xf numFmtId="0" fontId="11" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="165" fontId="14" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1643,7 +1643,7 @@
     <xf numFmtId="164" fontId="19" fillId="6" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="168" fontId="20" fillId="6" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="20" fillId="6" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1691,30 +1691,6 @@
     <xf numFmtId="0" fontId="21" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="21" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1788,6 +1764,42 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="4" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -2093,2080 +2105,2090 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:20" ht="19.5" thickBot="1">
-      <c r="A1" s="121" t="s">
+      <c r="A1" s="142" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="122"/>
-      <c r="C1" s="122"/>
-      <c r="D1" s="122"/>
-      <c r="E1" s="122"/>
-      <c r="F1" s="122"/>
-      <c r="G1" s="122"/>
-      <c r="H1" s="122"/>
-      <c r="I1" s="122"/>
-      <c r="J1" s="122"/>
-      <c r="K1" s="122"/>
-      <c r="L1" s="122"/>
-      <c r="M1" s="122"/>
-      <c r="N1" s="122"/>
-      <c r="O1" s="122"/>
-      <c r="P1" s="122"/>
-      <c r="Q1" s="122"/>
-      <c r="R1" s="122"/>
-      <c r="S1" s="122"/>
-      <c r="T1" s="123"/>
+      <c r="B1" s="143"/>
+      <c r="C1" s="143"/>
+      <c r="D1" s="143"/>
+      <c r="E1" s="143"/>
+      <c r="F1" s="143"/>
+      <c r="G1" s="143"/>
+      <c r="H1" s="143"/>
+      <c r="I1" s="143"/>
+      <c r="J1" s="143"/>
+      <c r="K1" s="143"/>
+      <c r="L1" s="143"/>
+      <c r="M1" s="143"/>
+      <c r="N1" s="143"/>
+      <c r="O1" s="143"/>
+      <c r="P1" s="143"/>
+      <c r="Q1" s="143"/>
+      <c r="R1" s="143"/>
+      <c r="S1" s="143"/>
+      <c r="T1" s="144"/>
     </row>
     <row r="2" spans="1:20" ht="16.5" thickBot="1">
-      <c r="A2" s="120" t="s">
+      <c r="A2" s="116" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="129" t="s">
+      <c r="B2" s="117" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="129" t="s">
+      <c r="C2" s="117" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="129" t="s">
+      <c r="D2" s="117" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="130" t="s">
+      <c r="E2" s="118" t="s">
         <v>5</v>
       </c>
-      <c r="F2" s="129" t="s">
+      <c r="F2" s="117" t="s">
         <v>6</v>
       </c>
-      <c r="G2" s="129" t="s">
+      <c r="G2" s="117" t="s">
         <v>7</v>
       </c>
-      <c r="H2" s="130" t="s">
+      <c r="H2" s="118" t="s">
         <v>8</v>
       </c>
-      <c r="I2" s="129" t="s">
+      <c r="I2" s="117" t="s">
         <v>9</v>
       </c>
-      <c r="J2" s="129" t="s">
+      <c r="J2" s="117" t="s">
         <v>10</v>
       </c>
-      <c r="K2" s="129" t="s">
+      <c r="K2" s="117" t="s">
         <v>11</v>
       </c>
-      <c r="L2" s="129" t="s">
+      <c r="L2" s="117" t="s">
         <v>12</v>
       </c>
-      <c r="M2" s="129" t="s">
+      <c r="M2" s="117" t="s">
         <v>13</v>
       </c>
-      <c r="N2" s="131" t="s">
+      <c r="N2" s="119" t="s">
         <v>14</v>
       </c>
-      <c r="O2" s="129" t="s">
+      <c r="O2" s="117" t="s">
         <v>15</v>
       </c>
-      <c r="P2" s="129" t="s">
+      <c r="P2" s="117" t="s">
         <v>16</v>
       </c>
-      <c r="Q2" s="129" t="s">
+      <c r="Q2" s="117" t="s">
         <v>17</v>
       </c>
-      <c r="R2" s="129" t="s">
+      <c r="R2" s="117" t="s">
         <v>18</v>
       </c>
-      <c r="S2" s="129" t="s">
+      <c r="S2" s="117" t="s">
         <v>19</v>
       </c>
-      <c r="T2" s="132" t="s">
+      <c r="T2" s="120" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="3" spans="1:20" ht="15.75" thickBot="1">
-      <c r="A3" s="152">
+      <c r="A3" s="140">
         <v>1</v>
       </c>
-      <c r="B3" s="126" t="s">
+      <c r="B3" s="147" t="s">
         <v>21</v>
       </c>
-      <c r="C3" s="9" t="s">
+      <c r="C3" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="D3" s="10" t="s">
+      <c r="D3" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="E3" s="10" t="s">
+      <c r="E3" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="F3" s="10" t="s">
+      <c r="F3" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="G3" s="10" t="s">
+      <c r="G3" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="H3" s="11" t="s">
+      <c r="H3" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="I3" s="12" t="s">
+      <c r="I3" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="J3" s="10" t="s">
+      <c r="J3" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="K3" s="50">
+      <c r="K3" s="48">
         <v>1</v>
       </c>
-      <c r="L3" s="50">
+      <c r="L3" s="48">
         <f>K3*5</f>
         <v>5</v>
       </c>
-      <c r="M3" s="108">
+      <c r="M3" s="104">
         <v>20</v>
       </c>
-      <c r="N3" s="109">
+      <c r="N3" s="105">
         <v>20</v>
       </c>
-      <c r="O3" s="52" t="s">
+      <c r="O3" s="50" t="s">
         <v>30</v>
       </c>
-      <c r="P3" s="53">
+      <c r="P3" s="51">
         <v>2.0299999999999999E-2</v>
       </c>
-      <c r="Q3" s="54">
+      <c r="Q3" s="52">
         <f>P3*M3</f>
         <v>0.40599999999999997</v>
       </c>
-      <c r="R3" s="53">
+      <c r="R3" s="51">
         <v>2.0299999999999999E-2</v>
       </c>
-      <c r="S3" s="54">
+      <c r="S3" s="52">
         <f>R3*N3</f>
         <v>0.40599999999999997</v>
       </c>
-      <c r="T3" s="55"/>
+      <c r="T3" s="53"/>
     </row>
     <row r="4" spans="1:20" ht="26.25" thickBot="1">
-      <c r="A4" s="152">
+      <c r="A4" s="140">
         <v>2</v>
       </c>
-      <c r="B4" s="124"/>
-      <c r="C4" s="13" t="s">
+      <c r="B4" s="148"/>
+      <c r="C4" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="D4" s="17" t="s">
+      <c r="D4" s="15" t="s">
         <v>32</v>
       </c>
-      <c r="E4" s="8" t="s">
+      <c r="E4" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="F4" s="8" t="s">
+      <c r="F4" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="G4" s="8" t="s">
+      <c r="G4" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="H4" s="133" t="s">
+      <c r="H4" s="121" t="s">
         <v>27</v>
       </c>
-      <c r="I4" s="14" t="s">
+      <c r="I4" s="12" t="s">
         <v>34</v>
       </c>
-      <c r="J4" s="8" t="s">
+      <c r="J4" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="K4" s="56">
+      <c r="K4" s="54">
         <v>20</v>
       </c>
-      <c r="L4" s="56">
+      <c r="L4" s="54">
         <f>K4*5</f>
         <v>100</v>
       </c>
-      <c r="M4" s="110">
+      <c r="M4" s="106">
         <v>100</v>
       </c>
-      <c r="N4" s="110">
+      <c r="N4" s="106">
         <v>200</v>
       </c>
-      <c r="O4" s="57" t="s">
+      <c r="O4" s="55" t="s">
         <v>30</v>
       </c>
-      <c r="P4" s="58">
+      <c r="P4" s="56">
         <v>2.8E-3</v>
       </c>
-      <c r="Q4" s="59">
+      <c r="Q4" s="57">
         <f t="shared" ref="Q4:Q34" si="0">P4*M4</f>
         <v>0.27999999999999997</v>
       </c>
-      <c r="R4" s="58">
+      <c r="R4" s="56">
         <v>2.8E-3</v>
       </c>
-      <c r="S4" s="59">
+      <c r="S4" s="57">
         <f t="shared" ref="S4:S34" si="1">R4*N4</f>
         <v>0.55999999999999994</v>
       </c>
-      <c r="T4" s="60"/>
+      <c r="T4" s="58"/>
     </row>
     <row r="5" spans="1:20" ht="15.75" thickBot="1">
-      <c r="A5" s="152">
+      <c r="A5" s="140">
         <v>3</v>
       </c>
-      <c r="B5" s="124"/>
-      <c r="C5" s="13" t="s">
+      <c r="B5" s="148"/>
+      <c r="C5" s="11" t="s">
         <v>36</v>
       </c>
-      <c r="D5" s="8" t="s">
+      <c r="D5" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="E5" s="8" t="s">
+      <c r="E5" s="6" t="s">
         <v>219</v>
       </c>
-      <c r="F5" s="8" t="s">
+      <c r="F5" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="G5" s="8" t="s">
+      <c r="G5" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="H5" s="133" t="s">
+      <c r="H5" s="121" t="s">
         <v>27</v>
       </c>
-      <c r="I5" s="8" t="s">
+      <c r="I5" s="6" t="s">
         <v>220</v>
       </c>
-      <c r="J5" s="8" t="s">
+      <c r="J5" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="K5" s="56">
+      <c r="K5" s="54">
         <v>1</v>
       </c>
-      <c r="L5" s="56">
+      <c r="L5" s="54">
         <f t="shared" ref="L5:L15" si="2">K5*5</f>
         <v>5</v>
       </c>
-      <c r="M5" s="110">
+      <c r="M5" s="106">
         <v>5</v>
       </c>
-      <c r="N5" s="110">
+      <c r="N5" s="106">
         <v>7</v>
       </c>
-      <c r="O5" s="57" t="s">
+      <c r="O5" s="55" t="s">
         <v>41</v>
       </c>
-      <c r="P5" s="61">
+      <c r="P5" s="59">
         <v>0.23400000000000001</v>
       </c>
-      <c r="Q5" s="59">
+      <c r="Q5" s="57">
         <f t="shared" si="0"/>
         <v>1.1700000000000002</v>
       </c>
-      <c r="R5" s="61">
+      <c r="R5" s="59">
         <v>0.23400000000000001</v>
       </c>
-      <c r="S5" s="59">
+      <c r="S5" s="57">
         <f t="shared" si="1"/>
         <v>1.6380000000000001</v>
       </c>
-      <c r="T5" s="60" t="s">
+      <c r="T5" s="58" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="6" spans="1:20" ht="15.75" thickBot="1">
-      <c r="A6" s="153">
+      <c r="A6" s="141">
         <v>4</v>
       </c>
-      <c r="B6" s="124"/>
-      <c r="C6" s="13" t="s">
+      <c r="B6" s="148"/>
+      <c r="C6" s="11" t="s">
         <v>43</v>
       </c>
-      <c r="D6" s="8" t="s">
+      <c r="D6" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="E6" s="8" t="s">
+      <c r="E6" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="F6" s="106" t="s">
+      <c r="F6" s="102" t="s">
         <v>46</v>
       </c>
-      <c r="G6" s="8" t="s">
+      <c r="G6" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="H6" s="133" t="s">
+      <c r="H6" s="121" t="s">
         <v>221</v>
       </c>
-      <c r="I6" s="15" t="s">
+      <c r="I6" s="13" t="s">
         <v>222</v>
       </c>
-      <c r="J6" s="8" t="s">
+      <c r="J6" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="K6" s="56">
+      <c r="K6" s="54">
         <v>2</v>
       </c>
-      <c r="L6" s="56">
+      <c r="L6" s="54">
         <f t="shared" si="2"/>
         <v>10</v>
       </c>
-      <c r="M6" s="110">
+      <c r="M6" s="106">
         <v>10</v>
       </c>
-      <c r="N6" s="110">
+      <c r="N6" s="106">
         <v>20</v>
       </c>
-      <c r="O6" s="107" t="s">
+      <c r="O6" s="103" t="s">
         <v>30</v>
       </c>
-      <c r="P6" s="58">
+      <c r="P6" s="56">
         <v>5.1799999999999999E-2</v>
       </c>
-      <c r="Q6" s="59">
+      <c r="Q6" s="57">
         <f t="shared" si="0"/>
         <v>0.51800000000000002</v>
       </c>
-      <c r="R6" s="58">
+      <c r="R6" s="56">
         <v>5.1799999999999999E-2</v>
       </c>
-      <c r="S6" s="59">
+      <c r="S6" s="57">
         <f t="shared" si="1"/>
         <v>1.036</v>
       </c>
-      <c r="T6" s="60"/>
+      <c r="T6" s="58"/>
     </row>
     <row r="7" spans="1:20" ht="15.75" thickBot="1">
-      <c r="A7" s="152">
+      <c r="A7" s="140">
         <v>5</v>
       </c>
-      <c r="B7" s="124"/>
-      <c r="C7" s="16" t="s">
+      <c r="B7" s="148"/>
+      <c r="C7" s="14" t="s">
         <v>49</v>
       </c>
-      <c r="D7" s="17" t="s">
+      <c r="D7" s="15" t="s">
         <v>50</v>
       </c>
-      <c r="E7" s="17" t="s">
+      <c r="E7" s="15" t="s">
         <v>45</v>
       </c>
-      <c r="F7" s="17" t="s">
+      <c r="F7" s="15" t="s">
         <v>51</v>
       </c>
-      <c r="G7" s="17" t="s">
+      <c r="G7" s="15" t="s">
         <v>52</v>
       </c>
-      <c r="H7" s="133" t="s">
+      <c r="H7" s="121" t="s">
         <v>27</v>
       </c>
-      <c r="I7" s="8" t="s">
+      <c r="I7" s="6" t="s">
         <v>223</v>
       </c>
-      <c r="J7" s="17" t="s">
+      <c r="J7" s="15" t="s">
         <v>53</v>
       </c>
-      <c r="K7" s="62">
+      <c r="K7" s="60">
         <v>2</v>
       </c>
-      <c r="L7" s="56">
+      <c r="L7" s="54">
         <f t="shared" si="2"/>
         <v>10</v>
       </c>
-      <c r="M7" s="110">
+      <c r="M7" s="106">
         <v>50</v>
       </c>
-      <c r="N7" s="110">
+      <c r="N7" s="106">
         <v>50</v>
       </c>
-      <c r="O7" s="63" t="s">
+      <c r="O7" s="61" t="s">
         <v>30</v>
       </c>
-      <c r="P7" s="58">
+      <c r="P7" s="56">
         <v>4.3E-3</v>
       </c>
-      <c r="Q7" s="59">
+      <c r="Q7" s="57">
         <f t="shared" si="0"/>
         <v>0.215</v>
       </c>
-      <c r="R7" s="58">
+      <c r="R7" s="56">
         <v>4.3E-3</v>
       </c>
-      <c r="S7" s="59">
+      <c r="S7" s="57">
         <f t="shared" si="1"/>
         <v>0.215</v>
       </c>
-      <c r="T7" s="60"/>
+      <c r="T7" s="58"/>
     </row>
     <row r="8" spans="1:20" ht="15.75" thickBot="1">
-      <c r="A8" s="152">
+      <c r="A8" s="140">
         <v>6</v>
       </c>
-      <c r="B8" s="124"/>
-      <c r="C8" s="13" t="s">
+      <c r="B8" s="148"/>
+      <c r="C8" s="11" t="s">
         <v>54</v>
       </c>
-      <c r="D8" s="8" t="s">
+      <c r="D8" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="E8" s="8" t="s">
+      <c r="E8" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="F8" s="106" t="s">
+      <c r="F8" s="102" t="s">
         <v>57</v>
       </c>
-      <c r="G8" s="8" t="s">
+      <c r="G8" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="H8" s="15" t="s">
+      <c r="H8" s="13" t="s">
         <v>59</v>
       </c>
-      <c r="I8" s="15" t="s">
+      <c r="I8" s="13" t="s">
         <v>60</v>
       </c>
-      <c r="J8" s="8" t="s">
+      <c r="J8" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="K8" s="56">
+      <c r="K8" s="54">
         <v>2</v>
       </c>
-      <c r="L8" s="56">
+      <c r="L8" s="54">
         <f t="shared" si="2"/>
         <v>10</v>
       </c>
-      <c r="M8" s="110">
+      <c r="M8" s="106">
         <v>100</v>
       </c>
-      <c r="N8" s="110">
+      <c r="N8" s="106">
         <v>100</v>
       </c>
-      <c r="O8" s="57" t="s">
+      <c r="O8" s="55" t="s">
         <v>30</v>
       </c>
-      <c r="P8" s="58">
+      <c r="P8" s="56">
         <v>3.3E-3</v>
       </c>
-      <c r="Q8" s="59">
+      <c r="Q8" s="57">
         <f t="shared" si="0"/>
         <v>0.33</v>
       </c>
-      <c r="R8" s="58">
+      <c r="R8" s="56">
         <v>3.3E-3</v>
       </c>
-      <c r="S8" s="59">
+      <c r="S8" s="57">
         <f t="shared" si="1"/>
         <v>0.33</v>
       </c>
-      <c r="T8" s="60"/>
+      <c r="T8" s="58"/>
     </row>
     <row r="9" spans="1:20" ht="15.75" thickBot="1">
-      <c r="A9" s="152">
+      <c r="A9" s="140">
         <v>7</v>
       </c>
-      <c r="B9" s="125"/>
-      <c r="C9" s="18" t="s">
+      <c r="B9" s="149"/>
+      <c r="C9" s="16" t="s">
         <v>62</v>
       </c>
-      <c r="D9" s="19" t="s">
+      <c r="D9" s="17" t="s">
         <v>63</v>
       </c>
-      <c r="E9" s="19" t="s">
+      <c r="E9" s="17" t="s">
         <v>24</v>
       </c>
-      <c r="F9" s="19" t="s">
+      <c r="F9" s="17" t="s">
         <v>64</v>
       </c>
-      <c r="G9" s="19" t="s">
+      <c r="G9" s="17" t="s">
         <v>26</v>
       </c>
-      <c r="H9" s="137" t="s">
+      <c r="H9" s="125" t="s">
         <v>27</v>
       </c>
-      <c r="I9" s="20" t="s">
+      <c r="I9" s="18" t="s">
         <v>65</v>
       </c>
-      <c r="J9" s="19" t="s">
+      <c r="J9" s="17" t="s">
         <v>66</v>
       </c>
-      <c r="K9" s="64">
+      <c r="K9" s="62">
         <v>1</v>
       </c>
-      <c r="L9" s="64">
+      <c r="L9" s="62">
         <f t="shared" si="2"/>
         <v>5</v>
       </c>
-      <c r="M9" s="112">
+      <c r="M9" s="108">
         <v>20</v>
       </c>
-      <c r="N9" s="112">
+      <c r="N9" s="108">
         <v>20</v>
       </c>
-      <c r="O9" s="111" t="s">
+      <c r="O9" s="107" t="s">
         <v>30</v>
       </c>
-      <c r="P9" s="66">
+      <c r="P9" s="64">
         <v>2.58E-2</v>
       </c>
-      <c r="Q9" s="67">
+      <c r="Q9" s="65">
         <f t="shared" si="0"/>
         <v>0.51600000000000001</v>
       </c>
-      <c r="R9" s="66">
+      <c r="R9" s="64">
         <v>2.58E-2</v>
       </c>
-      <c r="S9" s="67">
+      <c r="S9" s="65">
         <f t="shared" si="1"/>
         <v>0.51600000000000001</v>
       </c>
-      <c r="T9" s="68"/>
+      <c r="T9" s="66"/>
     </row>
     <row r="10" spans="1:20" ht="15.75" thickBot="1">
-      <c r="A10" s="152">
+      <c r="A10" s="140">
         <v>8</v>
       </c>
-      <c r="B10" s="126" t="s">
+      <c r="B10" s="147" t="s">
         <v>67</v>
       </c>
-      <c r="C10" s="21" t="s">
+      <c r="C10" s="19" t="s">
         <v>68</v>
       </c>
-      <c r="D10" s="22" t="s">
+      <c r="D10" s="20" t="s">
         <v>69</v>
       </c>
-      <c r="E10" s="22" t="s">
+      <c r="E10" s="20" t="s">
         <v>70</v>
       </c>
-      <c r="F10" s="22" t="s">
+      <c r="F10" s="20" t="s">
         <v>71</v>
       </c>
-      <c r="G10" s="22" t="s">
+      <c r="G10" s="20" t="s">
         <v>72</v>
       </c>
-      <c r="H10" s="23" t="s">
-        <v>27</v>
-      </c>
-      <c r="I10" s="23" t="s">
-        <v>27</v>
-      </c>
-      <c r="J10" s="24" t="s">
+      <c r="H10" s="21" t="s">
+        <v>230</v>
+      </c>
+      <c r="I10" s="21" t="s">
+        <v>231</v>
+      </c>
+      <c r="J10" s="22" t="s">
         <v>73</v>
       </c>
-      <c r="K10" s="69">
+      <c r="K10" s="67">
         <v>2</v>
       </c>
-      <c r="L10" s="69">
+      <c r="L10" s="67">
         <f t="shared" si="2"/>
         <v>10</v>
       </c>
-      <c r="M10" s="70"/>
-      <c r="N10" s="70"/>
-      <c r="O10" s="71"/>
-      <c r="P10" s="72"/>
-      <c r="Q10" s="73">
+      <c r="M10" s="153">
+        <v>50</v>
+      </c>
+      <c r="N10" s="153">
+        <v>50</v>
+      </c>
+      <c r="O10" s="152" t="s">
+        <v>30</v>
+      </c>
+      <c r="P10" s="68">
+        <v>1.49E-2</v>
+      </c>
+      <c r="Q10" s="69">
+        <f>P10*M10</f>
+        <v>0.745</v>
+      </c>
+      <c r="R10" s="68">
+        <v>1.49E-2</v>
+      </c>
+      <c r="S10" s="69">
+        <f t="shared" si="1"/>
+        <v>0.745</v>
+      </c>
+      <c r="T10" s="70" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="11" spans="1:20" ht="15.75" thickBot="1">
+      <c r="A11" s="140">
+        <v>9</v>
+      </c>
+      <c r="B11" s="148"/>
+      <c r="C11" s="11" t="s">
+        <v>75</v>
+      </c>
+      <c r="D11" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="E11" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="F11" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="G11" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="H11" s="6" t="s">
+        <v>224</v>
+      </c>
+      <c r="I11" s="13" t="s">
+        <v>225</v>
+      </c>
+      <c r="J11" s="122" t="s">
+        <v>73</v>
+      </c>
+      <c r="K11" s="54">
+        <v>1</v>
+      </c>
+      <c r="L11" s="54">
+        <f t="shared" si="2"/>
+        <v>5</v>
+      </c>
+      <c r="M11" s="106">
+        <v>5</v>
+      </c>
+      <c r="N11" s="106">
+        <v>10</v>
+      </c>
+      <c r="O11" s="103" t="s">
+        <v>30</v>
+      </c>
+      <c r="P11" s="59">
+        <v>9.9000000000000005E-2</v>
+      </c>
+      <c r="Q11" s="57">
+        <f t="shared" si="0"/>
+        <v>0.495</v>
+      </c>
+      <c r="R11" s="59">
+        <v>9.9000000000000005E-2</v>
+      </c>
+      <c r="S11" s="57">
+        <f t="shared" si="1"/>
+        <v>0.99</v>
+      </c>
+      <c r="T11" s="58"/>
+    </row>
+    <row r="12" spans="1:20" ht="15.75" thickBot="1">
+      <c r="A12" s="140">
+        <v>10</v>
+      </c>
+      <c r="B12" s="149"/>
+      <c r="C12" s="16" t="s">
+        <v>81</v>
+      </c>
+      <c r="D12" s="17" t="s">
+        <v>82</v>
+      </c>
+      <c r="E12" s="17" t="s">
+        <v>83</v>
+      </c>
+      <c r="F12" s="17" t="s">
+        <v>84</v>
+      </c>
+      <c r="G12" s="17" t="s">
+        <v>85</v>
+      </c>
+      <c r="H12" s="23" t="s">
+        <v>86</v>
+      </c>
+      <c r="I12" s="23" t="s">
+        <v>87</v>
+      </c>
+      <c r="J12" s="126" t="s">
+        <v>73</v>
+      </c>
+      <c r="K12" s="62">
+        <v>1</v>
+      </c>
+      <c r="L12" s="62">
+        <f t="shared" si="2"/>
+        <v>5</v>
+      </c>
+      <c r="M12" s="108">
+        <v>10</v>
+      </c>
+      <c r="N12" s="108">
+        <v>10</v>
+      </c>
+      <c r="O12" s="63" t="s">
+        <v>30</v>
+      </c>
+      <c r="P12" s="64">
+        <v>8.1699999999999995E-2</v>
+      </c>
+      <c r="Q12" s="65">
+        <f t="shared" si="0"/>
+        <v>0.81699999999999995</v>
+      </c>
+      <c r="R12" s="64">
+        <v>8.1699999999999995E-2</v>
+      </c>
+      <c r="S12" s="65">
+        <f t="shared" si="1"/>
+        <v>0.81699999999999995</v>
+      </c>
+      <c r="T12" s="66"/>
+    </row>
+    <row r="13" spans="1:20" ht="15.75" thickBot="1">
+      <c r="A13" s="140">
+        <v>11</v>
+      </c>
+      <c r="B13" s="150" t="s">
+        <v>88</v>
+      </c>
+      <c r="C13" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="D13" s="8" t="s">
+        <v>90</v>
+      </c>
+      <c r="E13" s="8" t="s">
+        <v>91</v>
+      </c>
+      <c r="F13" s="111" t="s">
+        <v>92</v>
+      </c>
+      <c r="G13" s="8" t="s">
+        <v>93</v>
+      </c>
+      <c r="H13" s="9" t="s">
+        <v>228</v>
+      </c>
+      <c r="I13" s="24" t="s">
+        <v>229</v>
+      </c>
+      <c r="J13" s="25" t="s">
+        <v>73</v>
+      </c>
+      <c r="K13" s="48">
+        <v>1</v>
+      </c>
+      <c r="L13" s="48">
+        <f t="shared" si="2"/>
+        <v>5</v>
+      </c>
+      <c r="M13" s="104">
+        <v>5</v>
+      </c>
+      <c r="N13" s="104">
+        <v>10</v>
+      </c>
+      <c r="O13" s="50" t="s">
+        <v>30</v>
+      </c>
+      <c r="P13" s="71">
+        <v>0.10630000000000001</v>
+      </c>
+      <c r="Q13" s="52">
+        <f t="shared" si="0"/>
+        <v>0.53150000000000008</v>
+      </c>
+      <c r="R13" s="71">
+        <v>0.10630000000000001</v>
+      </c>
+      <c r="S13" s="52">
+        <f t="shared" si="1"/>
+        <v>1.0630000000000002</v>
+      </c>
+      <c r="T13" s="53"/>
+    </row>
+    <row r="14" spans="1:20" ht="24.75" customHeight="1" thickBot="1">
+      <c r="A14" s="140">
+        <v>12</v>
+      </c>
+      <c r="B14" s="151"/>
+      <c r="C14" s="26" t="s">
+        <v>94</v>
+      </c>
+      <c r="D14" s="28" t="s">
+        <v>95</v>
+      </c>
+      <c r="E14" s="17" t="s">
+        <v>91</v>
+      </c>
+      <c r="F14" s="28" t="s">
+        <v>96</v>
+      </c>
+      <c r="G14" s="28" t="s">
+        <v>58</v>
+      </c>
+      <c r="H14" s="125" t="s">
+        <v>27</v>
+      </c>
+      <c r="I14" s="17" t="s">
+        <v>226</v>
+      </c>
+      <c r="J14" s="126" t="s">
+        <v>73</v>
+      </c>
+      <c r="K14" s="72">
+        <v>4</v>
+      </c>
+      <c r="L14" s="62">
+        <f t="shared" si="2"/>
+        <v>20</v>
+      </c>
+      <c r="M14" s="108">
+        <v>10</v>
+      </c>
+      <c r="N14" s="108">
+        <v>22</v>
+      </c>
+      <c r="O14" s="73" t="s">
+        <v>97</v>
+      </c>
+      <c r="P14" s="109">
+        <v>2.4029999999999999E-2</v>
+      </c>
+      <c r="Q14" s="65">
+        <f t="shared" si="0"/>
+        <v>0.24029999999999999</v>
+      </c>
+      <c r="R14" s="109">
+        <v>2.4029999999999999E-2</v>
+      </c>
+      <c r="S14" s="65">
+        <f t="shared" si="1"/>
+        <v>0.52866000000000002</v>
+      </c>
+      <c r="T14" s="66"/>
+    </row>
+    <row r="15" spans="1:20" ht="16.5" thickBot="1">
+      <c r="A15" s="140">
+        <v>13</v>
+      </c>
+      <c r="B15" s="138" t="s">
+        <v>98</v>
+      </c>
+      <c r="C15" s="137" t="s">
+        <v>99</v>
+      </c>
+      <c r="D15" s="127" t="s">
+        <v>100</v>
+      </c>
+      <c r="E15" s="127" t="s">
+        <v>101</v>
+      </c>
+      <c r="F15" s="127" t="s">
+        <v>102</v>
+      </c>
+      <c r="G15" s="127" t="s">
+        <v>103</v>
+      </c>
+      <c r="H15" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="I15" s="129" t="s">
+        <v>104</v>
+      </c>
+      <c r="J15" s="130" t="s">
+        <v>73</v>
+      </c>
+      <c r="K15" s="131">
+        <v>2</v>
+      </c>
+      <c r="L15" s="131">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
+      <c r="M15" s="132">
+        <v>20</v>
+      </c>
+      <c r="N15" s="132">
+        <v>20</v>
+      </c>
+      <c r="O15" s="133" t="s">
+        <v>30</v>
+      </c>
+      <c r="P15" s="134">
+        <v>5.0700000000000002E-2</v>
+      </c>
+      <c r="Q15" s="135">
+        <f t="shared" si="0"/>
+        <v>1.014</v>
+      </c>
+      <c r="R15" s="134">
+        <v>5.0700000000000002E-2</v>
+      </c>
+      <c r="S15" s="135">
+        <f t="shared" si="1"/>
+        <v>1.014</v>
+      </c>
+      <c r="T15" s="139"/>
+    </row>
+    <row r="16" spans="1:20" ht="51.75" thickBot="1">
+      <c r="A16" s="140">
+        <v>14</v>
+      </c>
+      <c r="B16" s="147" t="s">
+        <v>105</v>
+      </c>
+      <c r="C16" s="29" t="s">
+        <v>106</v>
+      </c>
+      <c r="D16" s="30" t="s">
+        <v>107</v>
+      </c>
+      <c r="E16" s="30" t="s">
+        <v>108</v>
+      </c>
+      <c r="F16" s="30" t="s">
+        <v>109</v>
+      </c>
+      <c r="G16" s="30" t="s">
+        <v>52</v>
+      </c>
+      <c r="H16" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="I16" s="31" t="s">
+        <v>110</v>
+      </c>
+      <c r="J16" s="30" t="s">
+        <v>111</v>
+      </c>
+      <c r="K16" s="74">
+        <v>40</v>
+      </c>
+      <c r="L16" s="48">
+        <f>K16*5</f>
+        <v>200</v>
+      </c>
+      <c r="M16" s="104">
+        <v>100</v>
+      </c>
+      <c r="N16" s="104">
+        <v>300</v>
+      </c>
+      <c r="O16" s="50" t="s">
+        <v>30</v>
+      </c>
+      <c r="P16" s="71">
+        <v>8.9999999999999998E-4</v>
+      </c>
+      <c r="Q16" s="52">
+        <f t="shared" si="0"/>
+        <v>0.09</v>
+      </c>
+      <c r="R16" s="71">
+        <v>8.9999999999999998E-4</v>
+      </c>
+      <c r="S16" s="52">
+        <f t="shared" si="1"/>
+        <v>0.27</v>
+      </c>
+      <c r="T16" s="53"/>
+    </row>
+    <row r="17" spans="1:20" ht="15.75" thickBot="1">
+      <c r="A17" s="140">
+        <v>15</v>
+      </c>
+      <c r="B17" s="148"/>
+      <c r="C17" s="11" t="s">
+        <v>112</v>
+      </c>
+      <c r="D17" s="47" t="s">
+        <v>113</v>
+      </c>
+      <c r="E17" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="F17" s="6" t="s">
+        <v>115</v>
+      </c>
+      <c r="G17" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="H17" s="121" t="s">
+        <v>27</v>
+      </c>
+      <c r="I17" s="13" t="s">
+        <v>116</v>
+      </c>
+      <c r="J17" s="6" t="s">
+        <v>117</v>
+      </c>
+      <c r="K17" s="54">
+        <v>7</v>
+      </c>
+      <c r="L17" s="54">
+        <f t="shared" ref="L17:L32" si="3">K17*5</f>
+        <v>35</v>
+      </c>
+      <c r="M17" s="106">
+        <v>100</v>
+      </c>
+      <c r="N17" s="106">
+        <v>100</v>
+      </c>
+      <c r="O17" s="55" t="s">
+        <v>30</v>
+      </c>
+      <c r="P17" s="56">
+        <v>1.2999999999999999E-3</v>
+      </c>
+      <c r="Q17" s="57">
+        <f t="shared" si="0"/>
+        <v>0.13</v>
+      </c>
+      <c r="R17" s="56">
+        <v>1.2999999999999999E-3</v>
+      </c>
+      <c r="S17" s="57">
+        <f t="shared" si="1"/>
+        <v>0.13</v>
+      </c>
+      <c r="T17" s="58"/>
+    </row>
+    <row r="18" spans="1:20" ht="15.75" thickBot="1">
+      <c r="A18" s="140">
+        <v>16</v>
+      </c>
+      <c r="B18" s="148"/>
+      <c r="C18" s="11" t="s">
+        <v>118</v>
+      </c>
+      <c r="D18" s="6" t="s">
+        <v>119</v>
+      </c>
+      <c r="E18" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="F18" s="6" t="s">
+        <v>120</v>
+      </c>
+      <c r="G18" s="110" t="s">
+        <v>121</v>
+      </c>
+      <c r="H18" s="13" t="s">
+        <v>122</v>
+      </c>
+      <c r="I18" s="13" t="s">
+        <v>123</v>
+      </c>
+      <c r="J18" s="6" t="s">
+        <v>124</v>
+      </c>
+      <c r="K18" s="54">
+        <v>1</v>
+      </c>
+      <c r="L18" s="54">
+        <f t="shared" si="3"/>
+        <v>5</v>
+      </c>
+      <c r="M18" s="106">
+        <v>100</v>
+      </c>
+      <c r="N18" s="106">
+        <v>100</v>
+      </c>
+      <c r="O18" s="55" t="s">
+        <v>30</v>
+      </c>
+      <c r="P18" s="59">
+        <v>2E-3</v>
+      </c>
+      <c r="Q18" s="57">
+        <f t="shared" si="0"/>
+        <v>0.2</v>
+      </c>
+      <c r="R18" s="59">
+        <v>2E-3</v>
+      </c>
+      <c r="S18" s="57">
+        <f t="shared" si="1"/>
+        <v>0.2</v>
+      </c>
+      <c r="T18" s="58"/>
+    </row>
+    <row r="19" spans="1:20" ht="15.75" thickBot="1">
+      <c r="A19" s="140">
+        <v>17</v>
+      </c>
+      <c r="B19" s="148"/>
+      <c r="C19" s="11" t="s">
+        <v>125</v>
+      </c>
+      <c r="D19" s="6" t="s">
+        <v>126</v>
+      </c>
+      <c r="E19" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="F19" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="G19" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="H19" s="121" t="s">
+        <v>27</v>
+      </c>
+      <c r="I19" s="13" t="s">
+        <v>128</v>
+      </c>
+      <c r="J19" s="6" t="s">
+        <v>129</v>
+      </c>
+      <c r="K19" s="54">
+        <v>2</v>
+      </c>
+      <c r="L19" s="54">
+        <f t="shared" si="3"/>
+        <v>10</v>
+      </c>
+      <c r="M19" s="106">
+        <v>100</v>
+      </c>
+      <c r="N19" s="106">
+        <v>100</v>
+      </c>
+      <c r="O19" s="55" t="s">
+        <v>30</v>
+      </c>
+      <c r="P19" s="59">
+        <v>1.4E-3</v>
+      </c>
+      <c r="Q19" s="57">
+        <f t="shared" si="0"/>
+        <v>0.13999999999999999</v>
+      </c>
+      <c r="R19" s="59">
+        <v>1.4E-3</v>
+      </c>
+      <c r="S19" s="57">
+        <f t="shared" si="1"/>
+        <v>0.13999999999999999</v>
+      </c>
+      <c r="T19" s="58"/>
+    </row>
+    <row r="20" spans="1:20" ht="15.75" thickBot="1">
+      <c r="A20" s="140">
+        <v>18</v>
+      </c>
+      <c r="B20" s="148"/>
+      <c r="C20" s="11" t="s">
+        <v>130</v>
+      </c>
+      <c r="D20" s="6" t="s">
+        <v>131</v>
+      </c>
+      <c r="E20" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="F20" s="6" t="s">
+        <v>132</v>
+      </c>
+      <c r="G20" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="H20" s="121" t="s">
+        <v>27</v>
+      </c>
+      <c r="I20" s="13" t="s">
+        <v>133</v>
+      </c>
+      <c r="J20" s="6" t="s">
+        <v>134</v>
+      </c>
+      <c r="K20" s="54">
+        <v>1</v>
+      </c>
+      <c r="L20" s="54">
+        <f t="shared" si="3"/>
+        <v>5</v>
+      </c>
+      <c r="M20" s="106">
+        <v>100</v>
+      </c>
+      <c r="N20" s="106">
+        <v>100</v>
+      </c>
+      <c r="O20" s="55" t="s">
+        <v>30</v>
+      </c>
+      <c r="P20" s="59">
+        <v>1.4E-3</v>
+      </c>
+      <c r="Q20" s="57">
+        <f t="shared" si="0"/>
+        <v>0.13999999999999999</v>
+      </c>
+      <c r="R20" s="59">
+        <v>1.4E-3</v>
+      </c>
+      <c r="S20" s="57">
+        <f t="shared" si="1"/>
+        <v>0.13999999999999999</v>
+      </c>
+      <c r="T20" s="58"/>
+    </row>
+    <row r="21" spans="1:20" ht="15.75" thickBot="1">
+      <c r="A21" s="140">
+        <v>19</v>
+      </c>
+      <c r="B21" s="149"/>
+      <c r="C21" s="16" t="s">
+        <v>135</v>
+      </c>
+      <c r="D21" s="17" t="s">
+        <v>136</v>
+      </c>
+      <c r="E21" s="17" t="s">
+        <v>114</v>
+      </c>
+      <c r="F21" s="17" t="s">
+        <v>137</v>
+      </c>
+      <c r="G21" s="17" t="s">
+        <v>52</v>
+      </c>
+      <c r="H21" s="125" t="s">
+        <v>27</v>
+      </c>
+      <c r="I21" s="27" t="s">
+        <v>138</v>
+      </c>
+      <c r="J21" s="17" t="s">
+        <v>139</v>
+      </c>
+      <c r="K21" s="62">
+        <v>2</v>
+      </c>
+      <c r="L21" s="62">
+        <f t="shared" si="3"/>
+        <v>10</v>
+      </c>
+      <c r="M21" s="108">
+        <v>50</v>
+      </c>
+      <c r="N21" s="108">
+        <v>50</v>
+      </c>
+      <c r="O21" s="63" t="s">
+        <v>30</v>
+      </c>
+      <c r="P21" s="64">
+        <v>4.7000000000000002E-3</v>
+      </c>
+      <c r="Q21" s="65">
+        <f t="shared" si="0"/>
+        <v>0.23500000000000001</v>
+      </c>
+      <c r="R21" s="64">
+        <v>4.7000000000000002E-3</v>
+      </c>
+      <c r="S21" s="65">
+        <f t="shared" si="1"/>
+        <v>0.23500000000000001</v>
+      </c>
+      <c r="T21" s="66"/>
+    </row>
+    <row r="22" spans="1:20" ht="16.5" thickBot="1">
+      <c r="A22" s="140">
+        <v>20</v>
+      </c>
+      <c r="B22" s="138" t="s">
+        <v>140</v>
+      </c>
+      <c r="C22" s="137" t="s">
+        <v>141</v>
+      </c>
+      <c r="D22" s="127" t="s">
+        <v>142</v>
+      </c>
+      <c r="E22" s="127" t="s">
+        <v>143</v>
+      </c>
+      <c r="F22" s="127" t="s">
+        <v>143</v>
+      </c>
+      <c r="G22" s="127" t="s">
+        <v>144</v>
+      </c>
+      <c r="H22" s="128" t="s">
+        <v>27</v>
+      </c>
+      <c r="I22" s="129" t="s">
+        <v>145</v>
+      </c>
+      <c r="J22" s="127" t="s">
+        <v>73</v>
+      </c>
+      <c r="K22" s="131">
+        <v>1</v>
+      </c>
+      <c r="L22" s="131">
+        <f t="shared" si="3"/>
+        <v>5</v>
+      </c>
+      <c r="M22" s="132">
+        <v>3</v>
+      </c>
+      <c r="N22" s="132">
+        <v>7</v>
+      </c>
+      <c r="O22" s="133" t="s">
+        <v>30</v>
+      </c>
+      <c r="P22" s="134">
+        <v>0.82230000000000003</v>
+      </c>
+      <c r="Q22" s="135">
+        <f t="shared" si="0"/>
+        <v>2.4668999999999999</v>
+      </c>
+      <c r="R22" s="134">
+        <v>0.82230000000000003</v>
+      </c>
+      <c r="S22" s="135">
+        <f t="shared" si="1"/>
+        <v>5.7561</v>
+      </c>
+      <c r="T22" s="139"/>
+    </row>
+    <row r="23" spans="1:20" ht="15.75" thickBot="1">
+      <c r="A23" s="140">
+        <v>21</v>
+      </c>
+      <c r="B23" s="147" t="s">
+        <v>146</v>
+      </c>
+      <c r="C23" s="7" t="s">
+        <v>147</v>
+      </c>
+      <c r="D23" s="8" t="s">
+        <v>148</v>
+      </c>
+      <c r="E23" s="8" t="s">
+        <v>213</v>
+      </c>
+      <c r="F23" s="8" t="s">
+        <v>149</v>
+      </c>
+      <c r="G23" s="8" t="s">
+        <v>150</v>
+      </c>
+      <c r="H23" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="I23" s="24" t="s">
+        <v>151</v>
+      </c>
+      <c r="J23" s="8" t="s">
+        <v>152</v>
+      </c>
+      <c r="K23" s="48">
+        <v>1</v>
+      </c>
+      <c r="L23" s="48">
+        <f t="shared" si="3"/>
+        <v>5</v>
+      </c>
+      <c r="M23" s="104">
+        <v>3</v>
+      </c>
+      <c r="N23" s="104">
+        <v>7</v>
+      </c>
+      <c r="O23" s="50" t="s">
+        <v>30</v>
+      </c>
+      <c r="P23" s="71">
+        <v>0.8458</v>
+      </c>
+      <c r="Q23" s="52">
+        <f t="shared" si="0"/>
+        <v>2.5373999999999999</v>
+      </c>
+      <c r="R23" s="71">
+        <v>0.8458</v>
+      </c>
+      <c r="S23" s="52">
+        <f t="shared" si="1"/>
+        <v>5.9206000000000003</v>
+      </c>
+      <c r="T23" s="53" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="24" spans="1:20" ht="15.75" thickBot="1">
+      <c r="A24" s="140">
+        <v>22</v>
+      </c>
+      <c r="B24" s="149"/>
+      <c r="C24" s="16" t="s">
+        <v>154</v>
+      </c>
+      <c r="D24" s="17" t="s">
+        <v>155</v>
+      </c>
+      <c r="E24" s="17" t="s">
+        <v>213</v>
+      </c>
+      <c r="F24" s="17" t="s">
+        <v>156</v>
+      </c>
+      <c r="G24" s="17" t="s">
+        <v>157</v>
+      </c>
+      <c r="H24" s="125" t="s">
+        <v>232</v>
+      </c>
+      <c r="I24" s="125" t="s">
+        <v>233</v>
+      </c>
+      <c r="J24" s="126" t="s">
+        <v>73</v>
+      </c>
+      <c r="K24" s="62">
+        <v>1</v>
+      </c>
+      <c r="L24" s="62">
+        <f t="shared" si="3"/>
+        <v>5</v>
+      </c>
+      <c r="M24" s="108">
+        <v>3</v>
+      </c>
+      <c r="N24" s="108">
+        <v>7</v>
+      </c>
+      <c r="O24" s="107" t="s">
+        <v>30</v>
+      </c>
+      <c r="P24" s="64">
+        <v>0.74480000000000002</v>
+      </c>
+      <c r="Q24" s="65">
+        <f t="shared" si="0"/>
+        <v>2.2343999999999999</v>
+      </c>
+      <c r="R24" s="64">
+        <v>0.74480000000000002</v>
+      </c>
+      <c r="S24" s="65">
+        <f t="shared" si="1"/>
+        <v>5.2136000000000005</v>
+      </c>
+      <c r="T24" s="66"/>
+    </row>
+    <row r="25" spans="1:20" ht="15.75" thickBot="1">
+      <c r="A25" s="140">
+        <v>23</v>
+      </c>
+      <c r="B25" s="147" t="s">
+        <v>158</v>
+      </c>
+      <c r="C25" s="32" t="s">
+        <v>159</v>
+      </c>
+      <c r="D25" s="33" t="s">
+        <v>160</v>
+      </c>
+      <c r="E25" s="33" t="s">
+        <v>161</v>
+      </c>
+      <c r="F25" s="33" t="s">
+        <v>162</v>
+      </c>
+      <c r="G25" s="33" t="s">
+        <v>163</v>
+      </c>
+      <c r="H25" s="34" t="s">
+        <v>27</v>
+      </c>
+      <c r="I25" s="34" t="s">
+        <v>27</v>
+      </c>
+      <c r="J25" s="35" t="s">
+        <v>73</v>
+      </c>
+      <c r="K25" s="75">
+        <v>1</v>
+      </c>
+      <c r="L25" s="76">
+        <f t="shared" si="3"/>
+        <v>5</v>
+      </c>
+      <c r="M25" s="77"/>
+      <c r="N25" s="78"/>
+      <c r="O25" s="79"/>
+      <c r="P25" s="80"/>
+      <c r="Q25" s="81">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="R10" s="72"/>
-      <c r="S10" s="73">
+      <c r="R25" s="80"/>
+      <c r="S25" s="81">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="T10" s="74" t="s">
-        <v>74</v>
+      <c r="T25" s="82" t="s">
+        <v>164</v>
       </c>
     </row>
-    <row r="11" spans="1:20" ht="15.75" thickBot="1">
-      <c r="A11" s="152">
-        <v>9</v>
-      </c>
-      <c r="B11" s="124"/>
-      <c r="C11" s="13" t="s">
-        <v>75</v>
-      </c>
-      <c r="D11" s="8" t="s">
-        <v>76</v>
-      </c>
-      <c r="E11" s="8" t="s">
-        <v>77</v>
-      </c>
-      <c r="F11" s="8" t="s">
-        <v>78</v>
-      </c>
-      <c r="G11" s="8" t="s">
-        <v>79</v>
-      </c>
-      <c r="H11" s="8" t="s">
-        <v>224</v>
-      </c>
-      <c r="I11" s="15" t="s">
-        <v>225</v>
-      </c>
-      <c r="J11" s="134" t="s">
+    <row r="26" spans="1:20" ht="15.75" thickBot="1">
+      <c r="A26" s="140">
+        <v>24</v>
+      </c>
+      <c r="B26" s="148"/>
+      <c r="C26" s="36" t="s">
+        <v>165</v>
+      </c>
+      <c r="D26" s="37" t="s">
+        <v>166</v>
+      </c>
+      <c r="E26" s="37" t="s">
+        <v>167</v>
+      </c>
+      <c r="F26" s="37" t="s">
+        <v>168</v>
+      </c>
+      <c r="G26" s="37" t="s">
+        <v>169</v>
+      </c>
+      <c r="H26" s="123" t="s">
+        <v>27</v>
+      </c>
+      <c r="I26" s="123" t="s">
+        <v>27</v>
+      </c>
+      <c r="J26" s="124" t="s">
         <v>73</v>
       </c>
-      <c r="K11" s="56">
+      <c r="K26" s="83">
         <v>1</v>
       </c>
-      <c r="L11" s="56">
-        <f t="shared" si="2"/>
-        <v>5</v>
-      </c>
-      <c r="M11" s="110">
-        <v>5</v>
-      </c>
-      <c r="N11" s="110">
-        <v>10</v>
-      </c>
-      <c r="O11" s="107" t="s">
-        <v>30</v>
-      </c>
-      <c r="P11" s="61">
-        <v>9.9000000000000005E-2</v>
-      </c>
-      <c r="Q11" s="59">
-        <f t="shared" si="0"/>
-        <v>0.495</v>
-      </c>
-      <c r="R11" s="61">
-        <v>9.9000000000000005E-2</v>
-      </c>
-      <c r="S11" s="59">
-        <f t="shared" si="1"/>
-        <v>0.99</v>
-      </c>
-      <c r="T11" s="60"/>
-    </row>
-    <row r="12" spans="1:20" ht="15.75" thickBot="1">
-      <c r="A12" s="152">
-        <v>10</v>
-      </c>
-      <c r="B12" s="125"/>
-      <c r="C12" s="18" t="s">
-        <v>81</v>
-      </c>
-      <c r="D12" s="19" t="s">
-        <v>82</v>
-      </c>
-      <c r="E12" s="19" t="s">
-        <v>83</v>
-      </c>
-      <c r="F12" s="19" t="s">
-        <v>84</v>
-      </c>
-      <c r="G12" s="19" t="s">
-        <v>85</v>
-      </c>
-      <c r="H12" s="25" t="s">
-        <v>86</v>
-      </c>
-      <c r="I12" s="25" t="s">
-        <v>87</v>
-      </c>
-      <c r="J12" s="138" t="s">
-        <v>73</v>
-      </c>
-      <c r="K12" s="64">
-        <v>1</v>
-      </c>
-      <c r="L12" s="64">
-        <f t="shared" si="2"/>
-        <v>5</v>
-      </c>
-      <c r="M12" s="112">
-        <v>10</v>
-      </c>
-      <c r="N12" s="112">
-        <v>10</v>
-      </c>
-      <c r="O12" s="65" t="s">
-        <v>30</v>
-      </c>
-      <c r="P12" s="66">
-        <v>8.1699999999999995E-2</v>
-      </c>
-      <c r="Q12" s="67">
-        <f t="shared" si="0"/>
-        <v>0.81699999999999995</v>
-      </c>
-      <c r="R12" s="66">
-        <v>8.1699999999999995E-2</v>
-      </c>
-      <c r="S12" s="67">
-        <f t="shared" si="1"/>
-        <v>0.81699999999999995</v>
-      </c>
-      <c r="T12" s="68"/>
-    </row>
-    <row r="13" spans="1:20" ht="15.75" thickBot="1">
-      <c r="A13" s="152">
-        <v>11</v>
-      </c>
-      <c r="B13" s="127" t="s">
-        <v>88</v>
-      </c>
-      <c r="C13" s="9" t="s">
-        <v>89</v>
-      </c>
-      <c r="D13" s="10" t="s">
-        <v>90</v>
-      </c>
-      <c r="E13" s="10" t="s">
-        <v>91</v>
-      </c>
-      <c r="F13" s="115" t="s">
-        <v>92</v>
-      </c>
-      <c r="G13" s="10" t="s">
-        <v>93</v>
-      </c>
-      <c r="H13" s="11" t="s">
-        <v>228</v>
-      </c>
-      <c r="I13" s="26" t="s">
-        <v>229</v>
-      </c>
-      <c r="J13" s="27" t="s">
-        <v>73</v>
-      </c>
-      <c r="K13" s="50">
-        <v>1</v>
-      </c>
-      <c r="L13" s="50">
-        <f t="shared" si="2"/>
-        <v>5</v>
-      </c>
-      <c r="M13" s="108">
-        <v>5</v>
-      </c>
-      <c r="N13" s="108">
-        <v>10</v>
-      </c>
-      <c r="O13" s="52" t="s">
-        <v>30</v>
-      </c>
-      <c r="P13" s="75">
-        <v>0.10630000000000001</v>
-      </c>
-      <c r="Q13" s="54">
-        <f t="shared" si="0"/>
-        <v>0.53150000000000008</v>
-      </c>
-      <c r="R13" s="75">
-        <v>0.10630000000000001</v>
-      </c>
-      <c r="S13" s="54">
-        <f t="shared" si="1"/>
-        <v>1.0630000000000002</v>
-      </c>
-      <c r="T13" s="55"/>
-    </row>
-    <row r="14" spans="1:20" ht="24.75" customHeight="1" thickBot="1">
-      <c r="A14" s="152">
-        <v>12</v>
-      </c>
-      <c r="B14" s="128"/>
-      <c r="C14" s="28" t="s">
-        <v>94</v>
-      </c>
-      <c r="D14" s="30" t="s">
-        <v>95</v>
-      </c>
-      <c r="E14" s="19" t="s">
-        <v>91</v>
-      </c>
-      <c r="F14" s="30" t="s">
-        <v>96</v>
-      </c>
-      <c r="G14" s="30" t="s">
-        <v>58</v>
-      </c>
-      <c r="H14" s="137" t="s">
-        <v>27</v>
-      </c>
-      <c r="I14" s="19" t="s">
-        <v>226</v>
-      </c>
-      <c r="J14" s="138" t="s">
-        <v>73</v>
-      </c>
-      <c r="K14" s="76">
-        <v>4</v>
-      </c>
-      <c r="L14" s="64">
-        <f t="shared" si="2"/>
-        <v>20</v>
-      </c>
-      <c r="M14" s="112">
-        <v>10</v>
-      </c>
-      <c r="N14" s="112">
-        <v>22</v>
-      </c>
-      <c r="O14" s="77" t="s">
-        <v>97</v>
-      </c>
-      <c r="P14" s="113">
-        <v>2.4029999999999999E-2</v>
-      </c>
-      <c r="Q14" s="67">
-        <f t="shared" si="0"/>
-        <v>0.24029999999999999</v>
-      </c>
-      <c r="R14" s="113">
-        <v>2.4029999999999999E-2</v>
-      </c>
-      <c r="S14" s="67">
-        <f t="shared" si="1"/>
-        <v>0.52866000000000002</v>
-      </c>
-      <c r="T14" s="68"/>
-    </row>
-    <row r="15" spans="1:20" ht="16.5" thickBot="1">
-      <c r="A15" s="152">
-        <v>13</v>
-      </c>
-      <c r="B15" s="150" t="s">
-        <v>98</v>
-      </c>
-      <c r="C15" s="149" t="s">
-        <v>99</v>
-      </c>
-      <c r="D15" s="139" t="s">
-        <v>100</v>
-      </c>
-      <c r="E15" s="139" t="s">
-        <v>101</v>
-      </c>
-      <c r="F15" s="139" t="s">
-        <v>102</v>
-      </c>
-      <c r="G15" s="139" t="s">
-        <v>103</v>
-      </c>
-      <c r="H15" s="140" t="s">
-        <v>27</v>
-      </c>
-      <c r="I15" s="141" t="s">
-        <v>104</v>
-      </c>
-      <c r="J15" s="142" t="s">
-        <v>73</v>
-      </c>
-      <c r="K15" s="143">
-        <v>2</v>
-      </c>
-      <c r="L15" s="143">
-        <f t="shared" si="2"/>
-        <v>10</v>
-      </c>
-      <c r="M15" s="144">
-        <v>20</v>
-      </c>
-      <c r="N15" s="144">
-        <v>20</v>
-      </c>
-      <c r="O15" s="145" t="s">
-        <v>30</v>
-      </c>
-      <c r="P15" s="146">
-        <v>5.0700000000000002E-2</v>
-      </c>
-      <c r="Q15" s="147">
-        <f t="shared" si="0"/>
-        <v>1.014</v>
-      </c>
-      <c r="R15" s="146">
-        <v>5.0700000000000002E-2</v>
-      </c>
-      <c r="S15" s="147">
-        <f t="shared" si="1"/>
-        <v>1.014</v>
-      </c>
-      <c r="T15" s="151"/>
-    </row>
-    <row r="16" spans="1:20" ht="51.75" thickBot="1">
-      <c r="A16" s="152">
-        <v>14</v>
-      </c>
-      <c r="B16" s="126" t="s">
-        <v>105</v>
-      </c>
-      <c r="C16" s="31" t="s">
-        <v>106</v>
-      </c>
-      <c r="D16" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="E16" s="32" t="s">
-        <v>108</v>
-      </c>
-      <c r="F16" s="32" t="s">
-        <v>109</v>
-      </c>
-      <c r="G16" s="32" t="s">
-        <v>52</v>
-      </c>
-      <c r="H16" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="I16" s="33" t="s">
-        <v>110</v>
-      </c>
-      <c r="J16" s="32" t="s">
-        <v>111</v>
-      </c>
-      <c r="K16" s="78">
-        <v>40</v>
-      </c>
-      <c r="L16" s="50">
-        <f>K16*5</f>
-        <v>200</v>
-      </c>
-      <c r="M16" s="108">
-        <v>100</v>
-      </c>
-      <c r="N16" s="108">
-        <v>300</v>
-      </c>
-      <c r="O16" s="52" t="s">
-        <v>30</v>
-      </c>
-      <c r="P16" s="75">
-        <v>8.9999999999999998E-4</v>
-      </c>
-      <c r="Q16" s="54">
-        <f t="shared" si="0"/>
-        <v>0.09</v>
-      </c>
-      <c r="R16" s="75">
-        <v>8.9999999999999998E-4</v>
-      </c>
-      <c r="S16" s="54">
-        <f t="shared" si="1"/>
-        <v>0.27</v>
-      </c>
-      <c r="T16" s="55"/>
-    </row>
-    <row r="17" spans="1:20" ht="15.75" thickBot="1">
-      <c r="A17" s="152">
-        <v>15</v>
-      </c>
-      <c r="B17" s="124"/>
-      <c r="C17" s="13" t="s">
-        <v>112</v>
-      </c>
-      <c r="D17" s="49" t="s">
-        <v>113</v>
-      </c>
-      <c r="E17" s="8" t="s">
-        <v>114</v>
-      </c>
-      <c r="F17" s="8" t="s">
-        <v>115</v>
-      </c>
-      <c r="G17" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="H17" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="I17" s="15" t="s">
-        <v>116</v>
-      </c>
-      <c r="J17" s="8" t="s">
-        <v>117</v>
-      </c>
-      <c r="K17" s="56">
-        <v>7</v>
-      </c>
-      <c r="L17" s="56">
-        <f t="shared" ref="L17:L32" si="3">K17*5</f>
-        <v>35</v>
-      </c>
-      <c r="M17" s="110">
-        <v>100</v>
-      </c>
-      <c r="N17" s="110">
-        <v>100</v>
-      </c>
-      <c r="O17" s="57" t="s">
-        <v>30</v>
-      </c>
-      <c r="P17" s="58">
-        <v>1.2999999999999999E-3</v>
-      </c>
-      <c r="Q17" s="59">
-        <f t="shared" si="0"/>
-        <v>0.13</v>
-      </c>
-      <c r="R17" s="58">
-        <v>1.2999999999999999E-3</v>
-      </c>
-      <c r="S17" s="59">
-        <f t="shared" si="1"/>
-        <v>0.13</v>
-      </c>
-      <c r="T17" s="60"/>
-    </row>
-    <row r="18" spans="1:20" ht="15.75" thickBot="1">
-      <c r="A18" s="152">
-        <v>16</v>
-      </c>
-      <c r="B18" s="124"/>
-      <c r="C18" s="13" t="s">
-        <v>118</v>
-      </c>
-      <c r="D18" s="8" t="s">
-        <v>119</v>
-      </c>
-      <c r="E18" s="8" t="s">
-        <v>108</v>
-      </c>
-      <c r="F18" s="8" t="s">
-        <v>120</v>
-      </c>
-      <c r="G18" s="114" t="s">
-        <v>121</v>
-      </c>
-      <c r="H18" s="15" t="s">
-        <v>122</v>
-      </c>
-      <c r="I18" s="15" t="s">
-        <v>123</v>
-      </c>
-      <c r="J18" s="8" t="s">
-        <v>124</v>
-      </c>
-      <c r="K18" s="56">
-        <v>1</v>
-      </c>
-      <c r="L18" s="56">
+      <c r="L26" s="84">
         <f t="shared" si="3"/>
         <v>5</v>
       </c>
-      <c r="M18" s="110">
-        <v>100</v>
-      </c>
-      <c r="N18" s="110">
-        <v>100</v>
-      </c>
-      <c r="O18" s="57" t="s">
-        <v>30</v>
-      </c>
-      <c r="P18" s="61">
-        <v>2E-3</v>
-      </c>
-      <c r="Q18" s="59">
+      <c r="M26" s="85"/>
+      <c r="N26" s="86"/>
+      <c r="O26" s="87"/>
+      <c r="P26" s="88"/>
+      <c r="Q26" s="88">
         <f t="shared" si="0"/>
-        <v>0.2</v>
-      </c>
-      <c r="R18" s="61">
-        <v>2E-3</v>
-      </c>
-      <c r="S18" s="59">
+        <v>0</v>
+      </c>
+      <c r="R26" s="88"/>
+      <c r="S26" s="88">
         <f t="shared" si="1"/>
-        <v>0.2</v>
-      </c>
-      <c r="T18" s="60"/>
+        <v>0</v>
+      </c>
+      <c r="T26" s="89" t="s">
+        <v>164</v>
+      </c>
     </row>
-    <row r="19" spans="1:20" ht="15.75" thickBot="1">
-      <c r="A19" s="152">
-        <v>17</v>
-      </c>
-      <c r="B19" s="124"/>
-      <c r="C19" s="13" t="s">
-        <v>125</v>
-      </c>
-      <c r="D19" s="8" t="s">
-        <v>126</v>
-      </c>
-      <c r="E19" s="8" t="s">
-        <v>114</v>
-      </c>
-      <c r="F19" s="8" t="s">
-        <v>127</v>
-      </c>
-      <c r="G19" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="H19" s="133" t="s">
+    <row r="27" spans="1:20" ht="15.75" thickBot="1">
+      <c r="A27" s="140">
+        <v>25</v>
+      </c>
+      <c r="B27" s="148"/>
+      <c r="C27" s="11" t="s">
+        <v>170</v>
+      </c>
+      <c r="D27" s="6" t="s">
+        <v>171</v>
+      </c>
+      <c r="E27" s="6" t="s">
+        <v>172</v>
+      </c>
+      <c r="F27" s="6" t="s">
+        <v>173</v>
+      </c>
+      <c r="G27" s="6" t="s">
+        <v>174</v>
+      </c>
+      <c r="H27" s="121" t="s">
         <v>27</v>
       </c>
-      <c r="I19" s="15" t="s">
-        <v>128</v>
-      </c>
-      <c r="J19" s="8" t="s">
-        <v>129</v>
-      </c>
-      <c r="K19" s="56">
-        <v>2</v>
-      </c>
-      <c r="L19" s="56">
-        <f t="shared" si="3"/>
-        <v>10</v>
-      </c>
-      <c r="M19" s="110">
-        <v>100</v>
-      </c>
-      <c r="N19" s="110">
-        <v>100</v>
-      </c>
-      <c r="O19" s="57" t="s">
-        <v>30</v>
-      </c>
-      <c r="P19" s="61">
-        <v>1.4E-3</v>
-      </c>
-      <c r="Q19" s="59">
-        <f t="shared" si="0"/>
-        <v>0.13999999999999999</v>
-      </c>
-      <c r="R19" s="61">
-        <v>1.4E-3</v>
-      </c>
-      <c r="S19" s="59">
-        <f t="shared" si="1"/>
-        <v>0.13999999999999999</v>
-      </c>
-      <c r="T19" s="60"/>
-    </row>
-    <row r="20" spans="1:20" ht="15.75" thickBot="1">
-      <c r="A20" s="152">
-        <v>18</v>
-      </c>
-      <c r="B20" s="124"/>
-      <c r="C20" s="13" t="s">
-        <v>130</v>
-      </c>
-      <c r="D20" s="8" t="s">
-        <v>131</v>
-      </c>
-      <c r="E20" s="8" t="s">
-        <v>114</v>
-      </c>
-      <c r="F20" s="8" t="s">
-        <v>132</v>
-      </c>
-      <c r="G20" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="H20" s="133" t="s">
+      <c r="I27" s="121" t="s">
         <v>27</v>
       </c>
-      <c r="I20" s="15" t="s">
-        <v>133</v>
-      </c>
-      <c r="J20" s="8" t="s">
-        <v>134</v>
-      </c>
-      <c r="K20" s="56">
+      <c r="J27" s="122" t="s">
+        <v>73</v>
+      </c>
+      <c r="K27" s="54">
         <v>1</v>
       </c>
-      <c r="L20" s="56">
+      <c r="L27" s="54">
         <f t="shared" si="3"/>
         <v>5</v>
       </c>
-      <c r="M20" s="110">
-        <v>100</v>
-      </c>
-      <c r="N20" s="110">
-        <v>100</v>
-      </c>
-      <c r="O20" s="57" t="s">
-        <v>30</v>
-      </c>
-      <c r="P20" s="61">
-        <v>1.4E-3</v>
-      </c>
-      <c r="Q20" s="59">
+      <c r="M27" s="106">
+        <v>1</v>
+      </c>
+      <c r="N27" s="106">
+        <v>6</v>
+      </c>
+      <c r="O27" s="103" t="s">
+        <v>227</v>
+      </c>
+      <c r="P27" s="56">
+        <v>7.6</v>
+      </c>
+      <c r="Q27" s="57">
         <f t="shared" si="0"/>
-        <v>0.13999999999999999</v>
-      </c>
-      <c r="R20" s="61">
-        <v>1.4E-3</v>
-      </c>
-      <c r="S20" s="59">
+        <v>7.6</v>
+      </c>
+      <c r="R27" s="56">
+        <v>7.6</v>
+      </c>
+      <c r="S27" s="57">
         <f t="shared" si="1"/>
-        <v>0.13999999999999999</v>
-      </c>
-      <c r="T20" s="60"/>
+        <v>45.599999999999994</v>
+      </c>
+      <c r="T27" s="58" t="s">
+        <v>175</v>
+      </c>
     </row>
-    <row r="21" spans="1:20" ht="15.75" thickBot="1">
-      <c r="A21" s="152">
-        <v>19</v>
-      </c>
-      <c r="B21" s="125"/>
-      <c r="C21" s="18" t="s">
-        <v>135</v>
-      </c>
-      <c r="D21" s="19" t="s">
-        <v>136</v>
-      </c>
-      <c r="E21" s="19" t="s">
-        <v>114</v>
-      </c>
-      <c r="F21" s="19" t="s">
-        <v>137</v>
-      </c>
-      <c r="G21" s="19" t="s">
-        <v>52</v>
-      </c>
-      <c r="H21" s="137" t="s">
+    <row r="28" spans="1:20" ht="15.75" thickBot="1">
+      <c r="A28" s="140">
+        <v>26</v>
+      </c>
+      <c r="B28" s="148"/>
+      <c r="C28" s="11" t="s">
+        <v>176</v>
+      </c>
+      <c r="D28" s="6" t="s">
+        <v>177</v>
+      </c>
+      <c r="E28" s="6" t="s">
+        <v>178</v>
+      </c>
+      <c r="F28" s="6" t="s">
+        <v>179</v>
+      </c>
+      <c r="G28" s="6" t="s">
+        <v>180</v>
+      </c>
+      <c r="H28" s="121" t="s">
         <v>27</v>
       </c>
-      <c r="I21" s="29" t="s">
-        <v>138</v>
-      </c>
-      <c r="J21" s="19" t="s">
-        <v>139</v>
-      </c>
-      <c r="K21" s="64">
-        <v>2</v>
-      </c>
-      <c r="L21" s="64">
-        <f t="shared" si="3"/>
-        <v>10</v>
-      </c>
-      <c r="M21" s="112">
-        <v>50</v>
-      </c>
-      <c r="N21" s="112">
-        <v>50</v>
-      </c>
-      <c r="O21" s="65" t="s">
-        <v>30</v>
-      </c>
-      <c r="P21" s="66">
-        <v>4.7000000000000002E-3</v>
-      </c>
-      <c r="Q21" s="67">
-        <f t="shared" si="0"/>
-        <v>0.23500000000000001</v>
-      </c>
-      <c r="R21" s="66">
-        <v>4.7000000000000002E-3</v>
-      </c>
-      <c r="S21" s="67">
-        <f t="shared" si="1"/>
-        <v>0.23500000000000001</v>
-      </c>
-      <c r="T21" s="68"/>
-    </row>
-    <row r="22" spans="1:20" ht="16.5" thickBot="1">
-      <c r="A22" s="152">
-        <v>20</v>
-      </c>
-      <c r="B22" s="150" t="s">
-        <v>140</v>
-      </c>
-      <c r="C22" s="149" t="s">
-        <v>141</v>
-      </c>
-      <c r="D22" s="139" t="s">
-        <v>142</v>
-      </c>
-      <c r="E22" s="139" t="s">
-        <v>143</v>
-      </c>
-      <c r="F22" s="139" t="s">
-        <v>143</v>
-      </c>
-      <c r="G22" s="139" t="s">
-        <v>144</v>
-      </c>
-      <c r="H22" s="140" t="s">
+      <c r="I28" s="121" t="s">
         <v>27</v>
       </c>
-      <c r="I22" s="141" t="s">
-        <v>145</v>
-      </c>
-      <c r="J22" s="139" t="s">
+      <c r="J28" s="122" t="s">
         <v>73</v>
       </c>
-      <c r="K22" s="143">
+      <c r="K28" s="54">
         <v>1</v>
       </c>
-      <c r="L22" s="143">
+      <c r="L28" s="54">
         <f t="shared" si="3"/>
         <v>5</v>
       </c>
-      <c r="M22" s="144">
-        <v>3</v>
-      </c>
-      <c r="N22" s="144">
-        <v>7</v>
-      </c>
-      <c r="O22" s="145" t="s">
-        <v>30</v>
-      </c>
-      <c r="P22" s="146">
-        <v>0.82230000000000003</v>
-      </c>
-      <c r="Q22" s="147">
+      <c r="M28" s="106">
+        <v>2</v>
+      </c>
+      <c r="N28" s="106">
+        <v>6</v>
+      </c>
+      <c r="O28" s="55" t="s">
+        <v>80</v>
+      </c>
+      <c r="P28" s="90">
+        <v>11</v>
+      </c>
+      <c r="Q28" s="57">
         <f t="shared" si="0"/>
-        <v>2.4668999999999999</v>
-      </c>
-      <c r="R22" s="146">
-        <v>0.82230000000000003</v>
-      </c>
-      <c r="S22" s="147">
+        <v>22</v>
+      </c>
+      <c r="R28" s="90">
+        <v>11</v>
+      </c>
+      <c r="S28" s="57">
         <f t="shared" si="1"/>
-        <v>5.7561</v>
-      </c>
-      <c r="T22" s="151"/>
+        <v>66</v>
+      </c>
+      <c r="T28" s="58"/>
     </row>
-    <row r="23" spans="1:20" ht="15.75" thickBot="1">
-      <c r="A23" s="152">
-        <v>21</v>
-      </c>
-      <c r="B23" s="126" t="s">
-        <v>146</v>
-      </c>
-      <c r="C23" s="9" t="s">
-        <v>147</v>
-      </c>
-      <c r="D23" s="10" t="s">
-        <v>148</v>
-      </c>
-      <c r="E23" s="10" t="s">
-        <v>213</v>
-      </c>
-      <c r="F23" s="10" t="s">
-        <v>149</v>
-      </c>
-      <c r="G23" s="10" t="s">
-        <v>150</v>
-      </c>
-      <c r="H23" s="11" t="s">
+    <row r="29" spans="1:20" ht="15.75" thickBot="1">
+      <c r="A29" s="140">
         <v>27</v>
       </c>
-      <c r="I23" s="26" t="s">
-        <v>151</v>
-      </c>
-      <c r="J23" s="10" t="s">
-        <v>152</v>
-      </c>
-      <c r="K23" s="50">
+      <c r="B29" s="148"/>
+      <c r="C29" s="11" t="s">
+        <v>181</v>
+      </c>
+      <c r="D29" s="6" t="s">
+        <v>182</v>
+      </c>
+      <c r="E29" s="6" t="s">
+        <v>183</v>
+      </c>
+      <c r="F29" s="6" t="s">
+        <v>184</v>
+      </c>
+      <c r="G29" s="6" t="s">
+        <v>169</v>
+      </c>
+      <c r="H29" s="121" t="s">
+        <v>27</v>
+      </c>
+      <c r="I29" s="13" t="s">
+        <v>185</v>
+      </c>
+      <c r="J29" s="122" t="s">
+        <v>73</v>
+      </c>
+      <c r="K29" s="54">
         <v>1</v>
       </c>
-      <c r="L23" s="50">
+      <c r="L29" s="54">
         <f t="shared" si="3"/>
         <v>5</v>
       </c>
-      <c r="M23" s="108">
-        <v>3</v>
-      </c>
-      <c r="N23" s="108">
-        <v>7</v>
-      </c>
-      <c r="O23" s="52" t="s">
+      <c r="M29" s="106">
+        <v>2</v>
+      </c>
+      <c r="N29" s="106">
+        <v>6</v>
+      </c>
+      <c r="O29" s="55" t="s">
         <v>30</v>
       </c>
-      <c r="P23" s="75">
-        <v>0.8458</v>
-      </c>
-      <c r="Q23" s="54">
+      <c r="P29" s="56">
+        <v>0.27710000000000001</v>
+      </c>
+      <c r="Q29" s="57">
         <f t="shared" si="0"/>
-        <v>2.5373999999999999</v>
-      </c>
-      <c r="R23" s="75">
-        <v>0.8458</v>
-      </c>
-      <c r="S23" s="54">
+        <v>0.55420000000000003</v>
+      </c>
+      <c r="R29" s="56">
+        <v>0.27710000000000001</v>
+      </c>
+      <c r="S29" s="57">
         <f t="shared" si="1"/>
-        <v>5.9206000000000003</v>
-      </c>
-      <c r="T23" s="55" t="s">
-        <v>153</v>
-      </c>
+        <v>1.6626000000000001</v>
+      </c>
+      <c r="T29" s="58"/>
     </row>
-    <row r="24" spans="1:20" ht="15.75" thickBot="1">
-      <c r="A24" s="152">
-        <v>22</v>
-      </c>
-      <c r="B24" s="125"/>
-      <c r="C24" s="18" t="s">
-        <v>154</v>
-      </c>
-      <c r="D24" s="19" t="s">
-        <v>155</v>
-      </c>
-      <c r="E24" s="19" t="s">
-        <v>213</v>
-      </c>
-      <c r="F24" s="19" t="s">
-        <v>156</v>
-      </c>
-      <c r="G24" s="19" t="s">
-        <v>157</v>
-      </c>
-      <c r="H24" s="137" t="s">
+    <row r="30" spans="1:20" ht="15.75" thickBot="1">
+      <c r="A30" s="140">
+        <v>28</v>
+      </c>
+      <c r="B30" s="148"/>
+      <c r="C30" s="112" t="s">
+        <v>186</v>
+      </c>
+      <c r="D30" s="113" t="s">
+        <v>187</v>
+      </c>
+      <c r="E30" s="113" t="s">
+        <v>188</v>
+      </c>
+      <c r="F30" s="113" t="s">
+        <v>189</v>
+      </c>
+      <c r="G30" s="113" t="s">
+        <v>190</v>
+      </c>
+      <c r="H30" s="124" t="s">
         <v>27</v>
       </c>
-      <c r="I24" s="137" t="s">
+      <c r="I30" s="124" t="s">
         <v>27</v>
       </c>
-      <c r="J24" s="138" t="s">
+      <c r="J30" s="124" t="s">
         <v>73</v>
       </c>
-      <c r="K24" s="64">
+      <c r="K30" s="84">
         <v>1</v>
       </c>
-      <c r="L24" s="64">
+      <c r="L30" s="84">
         <f t="shared" si="3"/>
         <v>5</v>
       </c>
-      <c r="M24" s="112">
-        <v>3</v>
-      </c>
-      <c r="N24" s="112">
-        <v>7</v>
-      </c>
-      <c r="O24" s="111" t="s">
-        <v>227</v>
-      </c>
-      <c r="P24" s="66">
-        <v>0.73</v>
-      </c>
-      <c r="Q24" s="67">
+      <c r="M30" s="86"/>
+      <c r="N30" s="86"/>
+      <c r="O30" s="114"/>
+      <c r="P30" s="115"/>
+      <c r="Q30" s="115">
         <f t="shared" si="0"/>
-        <v>2.19</v>
-      </c>
-      <c r="R24" s="66">
-        <v>0.73</v>
-      </c>
-      <c r="S24" s="67">
+        <v>0</v>
+      </c>
+      <c r="R30" s="115"/>
+      <c r="S30" s="115">
         <f t="shared" si="1"/>
-        <v>5.1099999999999994</v>
-      </c>
-      <c r="T24" s="68"/>
+        <v>0</v>
+      </c>
+      <c r="T30" s="89" t="s">
+        <v>164</v>
+      </c>
     </row>
-    <row r="25" spans="1:20" ht="15.75" thickBot="1">
-      <c r="A25" s="152">
-        <v>23</v>
-      </c>
-      <c r="B25" s="126" t="s">
-        <v>158</v>
-      </c>
-      <c r="C25" s="34" t="s">
-        <v>159</v>
-      </c>
-      <c r="D25" s="35" t="s">
-        <v>160</v>
-      </c>
-      <c r="E25" s="35" t="s">
-        <v>161</v>
-      </c>
-      <c r="F25" s="35" t="s">
-        <v>162</v>
-      </c>
-      <c r="G25" s="35" t="s">
-        <v>163</v>
-      </c>
-      <c r="H25" s="36" t="s">
+    <row r="31" spans="1:20" ht="15.75" thickBot="1">
+      <c r="A31" s="140">
+        <v>29</v>
+      </c>
+      <c r="B31" s="149"/>
+      <c r="C31" s="16" t="s">
+        <v>191</v>
+      </c>
+      <c r="D31" s="17" t="s">
+        <v>192</v>
+      </c>
+      <c r="E31" s="17" t="s">
+        <v>193</v>
+      </c>
+      <c r="F31" s="17" t="s">
+        <v>194</v>
+      </c>
+      <c r="G31" s="17" t="s">
+        <v>79</v>
+      </c>
+      <c r="H31" s="125" t="s">
         <v>27</v>
       </c>
-      <c r="I25" s="36" t="s">
-        <v>27</v>
-      </c>
-      <c r="J25" s="37" t="s">
+      <c r="I31" s="18" t="s">
+        <v>195</v>
+      </c>
+      <c r="J31" s="126" t="s">
         <v>73</v>
       </c>
-      <c r="K25" s="79">
+      <c r="K31" s="62">
         <v>1</v>
       </c>
-      <c r="L25" s="80">
+      <c r="L31" s="62">
         <f t="shared" si="3"/>
         <v>5</v>
       </c>
-      <c r="M25" s="81"/>
-      <c r="N25" s="82"/>
-      <c r="O25" s="83"/>
-      <c r="P25" s="84"/>
-      <c r="Q25" s="85">
+      <c r="M31" s="108">
+        <v>2</v>
+      </c>
+      <c r="N31" s="108">
+        <v>7</v>
+      </c>
+      <c r="O31" s="73" t="s">
+        <v>30</v>
+      </c>
+      <c r="P31" s="64">
+        <v>0.96120000000000005</v>
+      </c>
+      <c r="Q31" s="65">
+        <f t="shared" si="0"/>
+        <v>1.9224000000000001</v>
+      </c>
+      <c r="R31" s="64">
+        <v>0.96120000000000005</v>
+      </c>
+      <c r="S31" s="65">
+        <f t="shared" si="1"/>
+        <v>6.7284000000000006</v>
+      </c>
+      <c r="T31" s="66"/>
+    </row>
+    <row r="32" spans="1:20" ht="15.75" thickBot="1">
+      <c r="A32" s="140">
+        <v>30</v>
+      </c>
+      <c r="B32" s="147" t="s">
+        <v>196</v>
+      </c>
+      <c r="C32" s="29" t="s">
+        <v>197</v>
+      </c>
+      <c r="D32" s="30" t="s">
+        <v>198</v>
+      </c>
+      <c r="E32" s="24" t="s">
+        <v>213</v>
+      </c>
+      <c r="F32" s="30" t="s">
+        <v>199</v>
+      </c>
+      <c r="G32" s="30" t="s">
+        <v>200</v>
+      </c>
+      <c r="H32" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="I32" s="38" t="s">
+        <v>201</v>
+      </c>
+      <c r="J32" s="25" t="s">
+        <v>73</v>
+      </c>
+      <c r="K32" s="74">
+        <v>1</v>
+      </c>
+      <c r="L32" s="48">
+        <f t="shared" si="3"/>
+        <v>5</v>
+      </c>
+      <c r="M32" s="49">
+        <v>2</v>
+      </c>
+      <c r="N32" s="49">
+        <v>7</v>
+      </c>
+      <c r="O32" s="91" t="s">
+        <v>30</v>
+      </c>
+      <c r="P32" s="71">
+        <v>8.0299999999999996E-2</v>
+      </c>
+      <c r="Q32" s="52">
+        <f t="shared" si="0"/>
+        <v>0.16059999999999999</v>
+      </c>
+      <c r="R32" s="71">
+        <v>8.0299999999999996E-2</v>
+      </c>
+      <c r="S32" s="52">
+        <f t="shared" si="1"/>
+        <v>0.56209999999999993</v>
+      </c>
+      <c r="T32" s="53"/>
+    </row>
+    <row r="33" spans="1:20" ht="15.75" thickBot="1">
+      <c r="A33" s="140">
+        <v>31</v>
+      </c>
+      <c r="B33" s="148"/>
+      <c r="C33" s="39" t="s">
+        <v>202</v>
+      </c>
+      <c r="D33" s="37" t="s">
+        <v>203</v>
+      </c>
+      <c r="E33" s="40"/>
+      <c r="F33" s="37" t="s">
+        <v>204</v>
+      </c>
+      <c r="G33" s="37" t="s">
+        <v>205</v>
+      </c>
+      <c r="H33" s="123" t="s">
+        <v>27</v>
+      </c>
+      <c r="I33" s="123" t="s">
+        <v>27</v>
+      </c>
+      <c r="J33" s="124" t="s">
+        <v>73</v>
+      </c>
+      <c r="K33" s="83">
+        <v>1</v>
+      </c>
+      <c r="L33" s="83"/>
+      <c r="M33" s="85"/>
+      <c r="N33" s="85"/>
+      <c r="O33" s="87"/>
+      <c r="P33" s="92"/>
+      <c r="Q33" s="88">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="R25" s="84"/>
-      <c r="S25" s="85">
+      <c r="R33" s="92"/>
+      <c r="S33" s="88">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="T25" s="86" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="26" spans="1:20" ht="15.75" thickBot="1">
-      <c r="A26" s="152">
-        <v>24</v>
-      </c>
-      <c r="B26" s="124"/>
-      <c r="C26" s="38" t="s">
-        <v>165</v>
-      </c>
-      <c r="D26" s="39" t="s">
-        <v>166</v>
-      </c>
-      <c r="E26" s="39" t="s">
-        <v>167</v>
-      </c>
-      <c r="F26" s="39" t="s">
-        <v>168</v>
-      </c>
-      <c r="G26" s="39" t="s">
-        <v>169</v>
-      </c>
-      <c r="H26" s="135" t="s">
-        <v>27</v>
-      </c>
-      <c r="I26" s="135" t="s">
-        <v>27</v>
-      </c>
-      <c r="J26" s="136" t="s">
-        <v>73</v>
-      </c>
-      <c r="K26" s="87">
-        <v>1</v>
-      </c>
-      <c r="L26" s="88">
-        <f t="shared" si="3"/>
-        <v>5</v>
-      </c>
-      <c r="M26" s="89"/>
-      <c r="N26" s="90"/>
-      <c r="O26" s="91"/>
-      <c r="P26" s="92"/>
-      <c r="Q26" s="92">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="R26" s="92"/>
-      <c r="S26" s="92">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="T26" s="93" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="27" spans="1:20" ht="15.75" thickBot="1">
-      <c r="A27" s="152">
-        <v>25</v>
-      </c>
-      <c r="B27" s="124"/>
-      <c r="C27" s="13" t="s">
-        <v>170</v>
-      </c>
-      <c r="D27" s="8" t="s">
-        <v>171</v>
-      </c>
-      <c r="E27" s="8" t="s">
-        <v>172</v>
-      </c>
-      <c r="F27" s="8" t="s">
-        <v>173</v>
-      </c>
-      <c r="G27" s="8" t="s">
-        <v>174</v>
-      </c>
-      <c r="H27" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="I27" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="J27" s="134" t="s">
-        <v>73</v>
-      </c>
-      <c r="K27" s="56">
-        <v>1</v>
-      </c>
-      <c r="L27" s="56">
-        <f t="shared" si="3"/>
-        <v>5</v>
-      </c>
-      <c r="M27" s="110">
-        <v>1</v>
-      </c>
-      <c r="N27" s="110">
-        <v>6</v>
-      </c>
-      <c r="O27" s="107" t="s">
-        <v>227</v>
-      </c>
-      <c r="P27" s="58">
-        <v>7.6</v>
-      </c>
-      <c r="Q27" s="59">
-        <f t="shared" si="0"/>
-        <v>7.6</v>
-      </c>
-      <c r="R27" s="58">
-        <v>7.6</v>
-      </c>
-      <c r="S27" s="59">
-        <f t="shared" si="1"/>
-        <v>45.599999999999994</v>
-      </c>
-      <c r="T27" s="60" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="28" spans="1:20" ht="15.75" thickBot="1">
-      <c r="A28" s="152">
-        <v>26</v>
-      </c>
-      <c r="B28" s="124"/>
-      <c r="C28" s="13" t="s">
-        <v>176</v>
-      </c>
-      <c r="D28" s="8" t="s">
-        <v>177</v>
-      </c>
-      <c r="E28" s="8" t="s">
-        <v>178</v>
-      </c>
-      <c r="F28" s="8" t="s">
-        <v>179</v>
-      </c>
-      <c r="G28" s="8" t="s">
-        <v>180</v>
-      </c>
-      <c r="H28" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="I28" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="J28" s="134" t="s">
-        <v>73</v>
-      </c>
-      <c r="K28" s="56">
-        <v>1</v>
-      </c>
-      <c r="L28" s="56">
-        <f t="shared" si="3"/>
-        <v>5</v>
-      </c>
-      <c r="M28" s="110">
-        <v>2</v>
-      </c>
-      <c r="N28" s="110">
-        <v>6</v>
-      </c>
-      <c r="O28" s="57" t="s">
-        <v>80</v>
-      </c>
-      <c r="P28" s="94">
-        <v>11</v>
-      </c>
-      <c r="Q28" s="59">
-        <f t="shared" si="0"/>
-        <v>22</v>
-      </c>
-      <c r="R28" s="94">
-        <v>11</v>
-      </c>
-      <c r="S28" s="59">
-        <f t="shared" si="1"/>
-        <v>66</v>
-      </c>
-      <c r="T28" s="60"/>
-    </row>
-    <row r="29" spans="1:20" ht="15.75" thickBot="1">
-      <c r="A29" s="152">
-        <v>27</v>
-      </c>
-      <c r="B29" s="124"/>
-      <c r="C29" s="13" t="s">
-        <v>181</v>
-      </c>
-      <c r="D29" s="8" t="s">
-        <v>182</v>
-      </c>
-      <c r="E29" s="8" t="s">
-        <v>183</v>
-      </c>
-      <c r="F29" s="8" t="s">
-        <v>184</v>
-      </c>
-      <c r="G29" s="8" t="s">
-        <v>169</v>
-      </c>
-      <c r="H29" s="133" t="s">
-        <v>27</v>
-      </c>
-      <c r="I29" s="15" t="s">
-        <v>185</v>
-      </c>
-      <c r="J29" s="134" t="s">
-        <v>73</v>
-      </c>
-      <c r="K29" s="56">
-        <v>1</v>
-      </c>
-      <c r="L29" s="56">
-        <f t="shared" si="3"/>
-        <v>5</v>
-      </c>
-      <c r="M29" s="110">
-        <v>2</v>
-      </c>
-      <c r="N29" s="110">
-        <v>6</v>
-      </c>
-      <c r="O29" s="57" t="s">
-        <v>30</v>
-      </c>
-      <c r="P29" s="58">
-        <v>0.27710000000000001</v>
-      </c>
-      <c r="Q29" s="59">
-        <f t="shared" si="0"/>
-        <v>0.55420000000000003</v>
-      </c>
-      <c r="R29" s="58">
-        <v>0.27710000000000001</v>
-      </c>
-      <c r="S29" s="59">
-        <f t="shared" si="1"/>
-        <v>1.6626000000000001</v>
-      </c>
-      <c r="T29" s="60"/>
-    </row>
-    <row r="30" spans="1:20" ht="15.75" thickBot="1">
-      <c r="A30" s="152">
-        <v>28</v>
-      </c>
-      <c r="B30" s="124"/>
-      <c r="C30" s="116" t="s">
-        <v>186</v>
-      </c>
-      <c r="D30" s="117" t="s">
-        <v>187</v>
-      </c>
-      <c r="E30" s="117" t="s">
-        <v>188</v>
-      </c>
-      <c r="F30" s="117" t="s">
-        <v>189</v>
-      </c>
-      <c r="G30" s="117" t="s">
-        <v>190</v>
-      </c>
-      <c r="H30" s="136" t="s">
-        <v>27</v>
-      </c>
-      <c r="I30" s="136" t="s">
-        <v>27</v>
-      </c>
-      <c r="J30" s="136" t="s">
-        <v>73</v>
-      </c>
-      <c r="K30" s="88">
-        <v>1</v>
-      </c>
-      <c r="L30" s="88">
-        <f t="shared" si="3"/>
-        <v>5</v>
-      </c>
-      <c r="M30" s="90"/>
-      <c r="N30" s="90"/>
-      <c r="O30" s="118"/>
-      <c r="P30" s="119"/>
-      <c r="Q30" s="119">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="R30" s="119"/>
-      <c r="S30" s="119">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="T30" s="93" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="31" spans="1:20" ht="15.75" thickBot="1">
-      <c r="A31" s="152">
-        <v>29</v>
-      </c>
-      <c r="B31" s="125"/>
-      <c r="C31" s="18" t="s">
-        <v>191</v>
-      </c>
-      <c r="D31" s="19" t="s">
-        <v>192</v>
-      </c>
-      <c r="E31" s="19" t="s">
-        <v>193</v>
-      </c>
-      <c r="F31" s="19" t="s">
-        <v>194</v>
-      </c>
-      <c r="G31" s="19" t="s">
-        <v>79</v>
-      </c>
-      <c r="H31" s="137" t="s">
-        <v>27</v>
-      </c>
-      <c r="I31" s="20" t="s">
-        <v>195</v>
-      </c>
-      <c r="J31" s="138" t="s">
-        <v>73</v>
-      </c>
-      <c r="K31" s="64">
-        <v>1</v>
-      </c>
-      <c r="L31" s="64">
-        <f t="shared" si="3"/>
-        <v>5</v>
-      </c>
-      <c r="M31" s="112">
-        <v>2</v>
-      </c>
-      <c r="N31" s="112">
-        <v>7</v>
-      </c>
-      <c r="O31" s="77" t="s">
-        <v>30</v>
-      </c>
-      <c r="P31" s="66">
-        <v>0.96120000000000005</v>
-      </c>
-      <c r="Q31" s="67">
-        <f t="shared" si="0"/>
-        <v>1.9224000000000001</v>
-      </c>
-      <c r="R31" s="66">
-        <v>0.96120000000000005</v>
-      </c>
-      <c r="S31" s="67">
-        <f t="shared" si="1"/>
-        <v>6.7284000000000006</v>
-      </c>
-      <c r="T31" s="68"/>
-    </row>
-    <row r="32" spans="1:20" ht="15.75" thickBot="1">
-      <c r="A32" s="152">
-        <v>30</v>
-      </c>
-      <c r="B32" s="126" t="s">
-        <v>196</v>
-      </c>
-      <c r="C32" s="31" t="s">
-        <v>197</v>
-      </c>
-      <c r="D32" s="32" t="s">
-        <v>198</v>
-      </c>
-      <c r="E32" s="26" t="s">
-        <v>213</v>
-      </c>
-      <c r="F32" s="32" t="s">
-        <v>199</v>
-      </c>
-      <c r="G32" s="32" t="s">
-        <v>200</v>
-      </c>
-      <c r="H32" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="I32" s="40" t="s">
-        <v>201</v>
-      </c>
-      <c r="J32" s="27" t="s">
-        <v>73</v>
-      </c>
-      <c r="K32" s="78">
-        <v>1</v>
-      </c>
-      <c r="L32" s="50">
-        <f t="shared" si="3"/>
-        <v>5</v>
-      </c>
-      <c r="M32" s="51">
-        <v>2</v>
-      </c>
-      <c r="N32" s="51">
-        <v>7</v>
-      </c>
-      <c r="O32" s="95" t="s">
-        <v>30</v>
-      </c>
-      <c r="P32" s="75">
-        <v>8.0299999999999996E-2</v>
-      </c>
-      <c r="Q32" s="54">
-        <f t="shared" si="0"/>
-        <v>0.16059999999999999</v>
-      </c>
-      <c r="R32" s="75">
-        <v>8.0299999999999996E-2</v>
-      </c>
-      <c r="S32" s="54">
-        <f t="shared" si="1"/>
-        <v>0.56209999999999993</v>
-      </c>
-      <c r="T32" s="55"/>
-    </row>
-    <row r="33" spans="1:20" ht="15.75" thickBot="1">
-      <c r="A33" s="152">
-        <v>31</v>
-      </c>
-      <c r="B33" s="124"/>
-      <c r="C33" s="41" t="s">
-        <v>202</v>
-      </c>
-      <c r="D33" s="39" t="s">
-        <v>203</v>
-      </c>
-      <c r="E33" s="42"/>
-      <c r="F33" s="39" t="s">
-        <v>204</v>
-      </c>
-      <c r="G33" s="39" t="s">
-        <v>205</v>
-      </c>
-      <c r="H33" s="135" t="s">
-        <v>27</v>
-      </c>
-      <c r="I33" s="135" t="s">
-        <v>27</v>
-      </c>
-      <c r="J33" s="136" t="s">
-        <v>73</v>
-      </c>
-      <c r="K33" s="87">
-        <v>1</v>
-      </c>
-      <c r="L33" s="87"/>
-      <c r="M33" s="89"/>
-      <c r="N33" s="89"/>
-      <c r="O33" s="91"/>
-      <c r="P33" s="96"/>
-      <c r="Q33" s="92">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="R33" s="96"/>
-      <c r="S33" s="92">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="T33" s="93" t="s">
+      <c r="T33" s="89" t="s">
         <v>164</v>
       </c>
     </row>
     <row r="34" spans="1:20" ht="15.75" thickBot="1">
-      <c r="A34" s="152">
+      <c r="A34" s="140">
         <v>32</v>
       </c>
-      <c r="B34" s="124"/>
-      <c r="C34" s="43" t="s">
+      <c r="B34" s="148"/>
+      <c r="C34" s="41" t="s">
         <v>206</v>
       </c>
-      <c r="D34" s="44" t="s">
+      <c r="D34" s="42" t="s">
         <v>207</v>
       </c>
-      <c r="E34" s="44" t="s">
+      <c r="E34" s="42" t="s">
         <v>208</v>
       </c>
-      <c r="F34" s="44" t="s">
+      <c r="F34" s="42" t="s">
         <v>208</v>
       </c>
-      <c r="G34" s="44" t="s">
+      <c r="G34" s="42" t="s">
         <v>209</v>
       </c>
-      <c r="H34" s="133" t="s">
+      <c r="H34" s="121" t="s">
         <v>27</v>
       </c>
-      <c r="I34" s="133" t="s">
+      <c r="I34" s="121" t="s">
         <v>27</v>
       </c>
-      <c r="J34" s="134" t="s">
+      <c r="J34" s="122" t="s">
         <v>73</v>
       </c>
-      <c r="K34" s="97">
+      <c r="K34" s="93">
         <v>1</v>
       </c>
-      <c r="L34" s="97">
+      <c r="L34" s="93">
         <f>K34*5</f>
         <v>5</v>
       </c>
-      <c r="M34" s="98">
+      <c r="M34" s="94">
         <v>3</v>
       </c>
-      <c r="N34" s="98">
+      <c r="N34" s="94">
         <v>7</v>
       </c>
-      <c r="O34" s="99" t="s">
+      <c r="O34" s="95" t="s">
         <v>210</v>
       </c>
-      <c r="P34" s="59">
+      <c r="P34" s="57">
         <v>0.5</v>
       </c>
-      <c r="Q34" s="59">
+      <c r="Q34" s="57">
         <f t="shared" si="0"/>
         <v>1.5</v>
       </c>
-      <c r="R34" s="59">
+      <c r="R34" s="57">
         <v>0.5</v>
       </c>
-      <c r="S34" s="59">
+      <c r="S34" s="57">
         <f t="shared" si="1"/>
         <v>3.5</v>
       </c>
-      <c r="T34" s="100"/>
+      <c r="T34" s="96"/>
     </row>
     <row r="35" spans="1:20" ht="15.75" thickBot="1">
-      <c r="A35" s="152">
+      <c r="A35" s="140">
         <v>33</v>
       </c>
-      <c r="B35" s="125"/>
-      <c r="C35" s="45" t="s">
+      <c r="B35" s="149"/>
+      <c r="C35" s="43" t="s">
         <v>211</v>
       </c>
-      <c r="D35" s="148" t="s">
+      <c r="D35" s="136" t="s">
         <v>212</v>
       </c>
-      <c r="E35" s="46" t="s">
+      <c r="E35" s="44" t="s">
         <v>213</v>
       </c>
-      <c r="F35" s="46" t="s">
+      <c r="F35" s="44" t="s">
         <v>214</v>
       </c>
-      <c r="G35" s="47" t="s">
+      <c r="G35" s="45" t="s">
         <v>215</v>
       </c>
-      <c r="H35" s="47" t="s">
+      <c r="H35" s="45" t="s">
         <v>215</v>
       </c>
-      <c r="I35" s="48" t="s">
+      <c r="I35" s="46" t="s">
         <v>215</v>
       </c>
-      <c r="J35" s="47" t="s">
+      <c r="J35" s="45" t="s">
         <v>73</v>
       </c>
-      <c r="K35" s="101">
+      <c r="K35" s="97">
         <v>8</v>
       </c>
-      <c r="L35" s="102">
+      <c r="L35" s="98">
         <f>K35*5</f>
         <v>40</v>
       </c>
-      <c r="M35" s="103" t="s">
+      <c r="M35" s="99" t="s">
         <v>215</v>
       </c>
-      <c r="N35" s="104" t="s">
+      <c r="N35" s="100" t="s">
         <v>215</v>
       </c>
-      <c r="O35" s="103" t="s">
+      <c r="O35" s="99" t="s">
         <v>215</v>
       </c>
-      <c r="P35" s="104" t="s">
+      <c r="P35" s="100" t="s">
         <v>215</v>
       </c>
-      <c r="Q35" s="103" t="s">
+      <c r="Q35" s="99" t="s">
         <v>215</v>
       </c>
-      <c r="R35" s="104" t="s">
+      <c r="R35" s="100" t="s">
         <v>215</v>
       </c>
-      <c r="S35" s="103" t="s">
+      <c r="S35" s="99" t="s">
         <v>215</v>
       </c>
-      <c r="T35" s="105" t="s">
+      <c r="T35" s="101" t="s">
         <v>216</v>
       </c>
     </row>
@@ -4181,19 +4203,19 @@
       <c r="H36" s="1"/>
       <c r="I36" s="1"/>
       <c r="J36" s="1"/>
-      <c r="K36" s="6" t="s">
+      <c r="K36" s="145" t="s">
         <v>217</v>
       </c>
-      <c r="L36" s="6"/>
-      <c r="M36" s="6"/>
-      <c r="N36" s="6"/>
-      <c r="O36" s="6"/>
-      <c r="P36" s="6"/>
+      <c r="L36" s="145"/>
+      <c r="M36" s="145"/>
+      <c r="N36" s="145"/>
+      <c r="O36" s="145"/>
+      <c r="P36" s="145"/>
       <c r="Q36" s="1"/>
       <c r="R36" s="1"/>
       <c r="S36" s="3">
         <f>SUM(S3:S35)</f>
-        <v>151.06845999999999</v>
+        <v>151.91705999999996</v>
       </c>
       <c r="T36" s="1"/>
     </row>
@@ -4208,22 +4230,22 @@
       <c r="H37" s="1"/>
       <c r="I37" s="1"/>
       <c r="J37" s="1"/>
-      <c r="K37" s="7" t="s">
+      <c r="K37" s="146" t="s">
         <v>218</v>
       </c>
-      <c r="L37" s="7"/>
-      <c r="M37" s="7"/>
-      <c r="N37" s="7"/>
-      <c r="O37" s="7"/>
-      <c r="P37" s="7"/>
+      <c r="L37" s="146"/>
+      <c r="M37" s="146"/>
+      <c r="N37" s="146"/>
+      <c r="O37" s="146"/>
+      <c r="P37" s="146"/>
       <c r="Q37" s="4">
         <f>SUM(Q3:Q36)</f>
-        <v>48.399300000000004</v>
+        <v>49.188700000000004</v>
       </c>
       <c r="R37" s="1"/>
       <c r="S37" s="5">
         <f>S36/5</f>
-        <v>30.213691999999998</v>
+        <v>30.383411999999993</v>
       </c>
       <c r="T37" s="1"/>
     </row>
@@ -4341,12 +4363,13 @@
     <hyperlink ref="O6" r:id="rId22" xr:uid="{8063891C-DF0E-4834-856E-F39EEA1E167D}"/>
     <hyperlink ref="O9" r:id="rId23" xr:uid="{9C9612D2-C88A-41A7-8FD4-08A80F130732}"/>
     <hyperlink ref="O11" r:id="rId24" xr:uid="{95D93024-AED5-474A-A44C-1977D53D1EBB}"/>
-    <hyperlink ref="O24" r:id="rId25" xr:uid="{426A1C96-310D-4503-9657-A4FFE1141619}"/>
-    <hyperlink ref="O27" r:id="rId26" xr:uid="{CF4B4C61-8EF1-4B30-8745-7950502015AE}"/>
+    <hyperlink ref="O27" r:id="rId25" xr:uid="{CF4B4C61-8EF1-4B30-8745-7950502015AE}"/>
+    <hyperlink ref="O10" r:id="rId26" xr:uid="{F1701D03-7653-426C-ADD2-6E97EA6BB057}"/>
+    <hyperlink ref="O24" r:id="rId27" xr:uid="{B75F8E8E-BDCC-4D93-89E1-5420EB14BD4C}"/>
   </hyperlinks>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.30555555555555602" right="0.30555555555555602" top="0.30555555555555602" bottom="0.30555555555555602" header="0" footer="0"/>
-  <pageSetup scale="39" orientation="landscape" blackAndWhite="1" r:id="rId27"/>
+  <pageSetup scale="39" orientation="landscape" blackAndWhite="1" r:id="rId28"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>

</xml_diff>